<commit_message>
Update master list before rollout
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -1492,10 +1492,19 @@
     <t>DI</t>
   </si>
   <si>
+    <t>MRI Handicap Toilet</t>
+  </si>
+  <si>
+    <t>IR Handicap Toilet</t>
+  </si>
+  <si>
+    <t>X-Ray Handicap Toilet</t>
+  </si>
+  <si>
+    <t>AMU</t>
+  </si>
+  <si>
     <t>Handicap Toilet</t>
-  </si>
-  <si>
-    <t>AMU</t>
   </si>
   <si>
     <t>KU</t>
@@ -16552,13 +16561,13 @@
         <v>486</v>
       </c>
       <c r="B189" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C189" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="D189" s="1" t="s">
         <v>489</v>
-      </c>
-      <c r="D189" s="1" t="s">
-        <v>488</v>
       </c>
       <c r="E189" s="1">
         <v>188</v>
@@ -16593,13 +16602,13 @@
         <v>486</v>
       </c>
       <c r="B190" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C190" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="D190" s="1" t="s">
         <v>490</v>
-      </c>
-      <c r="D190" s="1" t="s">
-        <v>488</v>
       </c>
       <c r="E190" s="1">
         <v>189</v>
@@ -16634,13 +16643,13 @@
         <v>486</v>
       </c>
       <c r="B191" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C191" s="1" t="s">
         <v>491</v>
       </c>
       <c r="D191" s="1" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="E191" s="1">
         <v>190</v>
@@ -16675,13 +16684,13 @@
         <v>486</v>
       </c>
       <c r="B192" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C192" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="D192" s="1" t="s">
         <v>492</v>
-      </c>
-      <c r="D192" s="1" t="s">
-        <v>488</v>
       </c>
       <c r="E192" s="1">
         <v>191</v>
@@ -16716,13 +16725,13 @@
         <v>486</v>
       </c>
       <c r="B193" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C193" s="1" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D193" s="1" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="E193" s="1">
         <v>192</v>
@@ -16740,10 +16749,10 @@
         <v>14</v>
       </c>
       <c r="J193" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K193" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L193" s="2" t="s">
         <v>14</v>
@@ -16757,13 +16766,13 @@
         <v>486</v>
       </c>
       <c r="B194" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C194" s="1" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D194" s="1" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="E194" s="1">
         <v>193</v>
@@ -16781,10 +16790,10 @@
         <v>14</v>
       </c>
       <c r="J194" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K194" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L194" s="2" t="s">
         <v>14</v>
@@ -16801,10 +16810,10 @@
         <v>5</v>
       </c>
       <c r="C195" s="1" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="D195" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E195" s="1">
         <v>194</v>
@@ -16842,10 +16851,10 @@
         <v>5</v>
       </c>
       <c r="C196" s="1" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="D196" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E196" s="1">
         <v>195</v>
@@ -16883,10 +16892,10 @@
         <v>5</v>
       </c>
       <c r="C197" s="1" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="D197" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E197" s="1">
         <v>196</v>
@@ -16924,10 +16933,10 @@
         <v>5</v>
       </c>
       <c r="C198" s="1" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="D198" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E198" s="1">
         <v>197</v>
@@ -16965,10 +16974,10 @@
         <v>5</v>
       </c>
       <c r="C199" s="1" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="D199" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E199" s="1">
         <v>198</v>
@@ -17006,7 +17015,7 @@
         <v>5</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="D200" s="1" t="s">
         <v>502</v>
@@ -17047,7 +17056,7 @@
         <v>5</v>
       </c>
       <c r="C201" s="1" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="D201" s="1" t="s">
         <v>503</v>
@@ -17088,10 +17097,10 @@
         <v>5</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="D202" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E202" s="1">
         <v>201</v>
@@ -17129,10 +17138,10 @@
         <v>5</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="D203" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E203" s="1">
         <v>202</v>
@@ -17167,13 +17176,13 @@
         <v>486</v>
       </c>
       <c r="B204" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D204" s="1" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="E204" s="1">
         <v>203</v>
@@ -17208,13 +17217,13 @@
         <v>486</v>
       </c>
       <c r="B205" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C205" s="1" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D205" s="1" t="s">
-        <v>495</v>
+        <v>508</v>
       </c>
       <c r="E205" s="1">
         <v>204</v>
@@ -17252,10 +17261,10 @@
         <v>6</v>
       </c>
       <c r="C206" s="1" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D206" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E206" s="1">
         <v>205</v>
@@ -17293,10 +17302,10 @@
         <v>6</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D207" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E207" s="1">
         <v>206</v>
@@ -17334,10 +17343,10 @@
         <v>6</v>
       </c>
       <c r="C208" s="1" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D208" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E208" s="1">
         <v>207</v>
@@ -17375,10 +17384,10 @@
         <v>6</v>
       </c>
       <c r="C209" s="1" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D209" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E209" s="1">
         <v>208</v>
@@ -17416,10 +17425,10 @@
         <v>6</v>
       </c>
       <c r="C210" s="1" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D210" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E210" s="1">
         <v>209</v>
@@ -17457,7 +17466,7 @@
         <v>6</v>
       </c>
       <c r="C211" s="1" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="D211" s="1" t="s">
         <v>502</v>
@@ -17498,7 +17507,7 @@
         <v>6</v>
       </c>
       <c r="C212" s="1" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="D212" s="1" t="s">
         <v>503</v>
@@ -17539,10 +17548,10 @@
         <v>6</v>
       </c>
       <c r="C213" s="1" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="D213" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E213" s="1">
         <v>212</v>
@@ -17580,10 +17589,10 @@
         <v>6</v>
       </c>
       <c r="C214" s="1" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="D214" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E214" s="1">
         <v>213</v>
@@ -17618,13 +17627,13 @@
         <v>486</v>
       </c>
       <c r="B215" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C215" s="1" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D215" s="1" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="E215" s="1">
         <v>214</v>
@@ -17659,13 +17668,13 @@
         <v>486</v>
       </c>
       <c r="B216" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C216" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="D216" s="1" t="s">
         <v>508</v>
-      </c>
-      <c r="D216" s="1" t="s">
-        <v>495</v>
       </c>
       <c r="E216" s="1">
         <v>215</v>
@@ -17703,10 +17712,10 @@
         <v>7</v>
       </c>
       <c r="C217" s="1" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D217" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E217" s="1">
         <v>216</v>
@@ -17744,10 +17753,10 @@
         <v>7</v>
       </c>
       <c r="C218" s="1" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D218" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E218" s="1">
         <v>217</v>
@@ -17785,10 +17794,10 @@
         <v>7</v>
       </c>
       <c r="C219" s="1" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D219" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E219" s="1">
         <v>218</v>
@@ -17826,10 +17835,10 @@
         <v>7</v>
       </c>
       <c r="C220" s="1" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D220" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E220" s="1">
         <v>219</v>
@@ -17867,10 +17876,10 @@
         <v>7</v>
       </c>
       <c r="C221" s="1" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D221" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E221" s="1">
         <v>220</v>
@@ -17908,7 +17917,7 @@
         <v>7</v>
       </c>
       <c r="C222" s="1" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="D222" s="1" t="s">
         <v>502</v>
@@ -17949,7 +17958,7 @@
         <v>7</v>
       </c>
       <c r="C223" s="1" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="D223" s="1" t="s">
         <v>503</v>
@@ -17990,10 +17999,10 @@
         <v>7</v>
       </c>
       <c r="C224" s="1" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="D224" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E224" s="1">
         <v>223</v>
@@ -18031,10 +18040,10 @@
         <v>7</v>
       </c>
       <c r="C225" s="1" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="D225" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E225" s="1">
         <v>224</v>
@@ -18069,13 +18078,13 @@
         <v>486</v>
       </c>
       <c r="B226" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C226" s="1" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="D226" s="1" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="E226" s="1">
         <v>225</v>
@@ -18110,13 +18119,13 @@
         <v>486</v>
       </c>
       <c r="B227" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C227" s="1" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="D227" s="1" t="s">
-        <v>495</v>
+        <v>508</v>
       </c>
       <c r="E227" s="1">
         <v>226</v>
@@ -18154,10 +18163,10 @@
         <v>8</v>
       </c>
       <c r="C228" s="1" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D228" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E228" s="1">
         <v>227</v>
@@ -18195,10 +18204,10 @@
         <v>8</v>
       </c>
       <c r="C229" s="1" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D229" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E229" s="1">
         <v>228</v>
@@ -18236,10 +18245,10 @@
         <v>8</v>
       </c>
       <c r="C230" s="1" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D230" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E230" s="1">
         <v>229</v>
@@ -18277,10 +18286,10 @@
         <v>8</v>
       </c>
       <c r="C231" s="1" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D231" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E231" s="1">
         <v>230</v>
@@ -18318,10 +18327,10 @@
         <v>8</v>
       </c>
       <c r="C232" s="1" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D232" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E232" s="1">
         <v>231</v>
@@ -18359,7 +18368,7 @@
         <v>8</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D233" s="1" t="s">
         <v>502</v>
@@ -18400,7 +18409,7 @@
         <v>8</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D234" s="1" t="s">
         <v>503</v>
@@ -18441,10 +18450,10 @@
         <v>8</v>
       </c>
       <c r="C235" s="1" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="D235" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E235" s="1">
         <v>234</v>
@@ -18482,10 +18491,10 @@
         <v>8</v>
       </c>
       <c r="C236" s="1" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="D236" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E236" s="1">
         <v>235</v>
@@ -18520,13 +18529,13 @@
         <v>486</v>
       </c>
       <c r="B237" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C237" s="1" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D237" s="1" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="E237" s="1">
         <v>236</v>
@@ -18561,13 +18570,13 @@
         <v>486</v>
       </c>
       <c r="B238" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C238" s="1" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D238" s="1" t="s">
-        <v>495</v>
+        <v>508</v>
       </c>
       <c r="E238" s="1">
         <v>237</v>
@@ -18605,10 +18614,10 @@
         <v>9</v>
       </c>
       <c r="C239" s="1" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="D239" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E239" s="1">
         <v>238</v>
@@ -18646,10 +18655,10 @@
         <v>9</v>
       </c>
       <c r="C240" s="1" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="D240" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E240" s="1">
         <v>239</v>
@@ -18687,10 +18696,10 @@
         <v>9</v>
       </c>
       <c r="C241" s="1" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="D241" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E241" s="1">
         <v>240</v>
@@ -18728,10 +18737,10 @@
         <v>9</v>
       </c>
       <c r="C242" s="1" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="D242" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E242" s="1">
         <v>241</v>
@@ -18769,10 +18778,10 @@
         <v>9</v>
       </c>
       <c r="C243" s="1" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="D243" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E243" s="1">
         <v>242</v>
@@ -18810,7 +18819,7 @@
         <v>9</v>
       </c>
       <c r="C244" s="1" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D244" s="1" t="s">
         <v>502</v>
@@ -18851,7 +18860,7 @@
         <v>9</v>
       </c>
       <c r="C245" s="1" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D245" s="1" t="s">
         <v>503</v>
@@ -18892,10 +18901,10 @@
         <v>9</v>
       </c>
       <c r="C246" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="D246" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E246" s="1">
         <v>245</v>
@@ -18933,10 +18942,10 @@
         <v>9</v>
       </c>
       <c r="C247" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="D247" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E247" s="1">
         <v>246</v>
@@ -18971,13 +18980,13 @@
         <v>486</v>
       </c>
       <c r="B248" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C248" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="D248" s="1" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="E248" s="1">
         <v>247</v>
@@ -19012,13 +19021,13 @@
         <v>486</v>
       </c>
       <c r="B249" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C249" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="D249" s="1" t="s">
-        <v>495</v>
+        <v>508</v>
       </c>
       <c r="E249" s="1">
         <v>248</v>
@@ -19056,10 +19065,10 @@
         <v>10</v>
       </c>
       <c r="C250" s="1" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D250" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E250" s="1">
         <v>249</v>
@@ -19097,10 +19106,10 @@
         <v>10</v>
       </c>
       <c r="C251" s="1" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D251" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E251" s="1">
         <v>250</v>
@@ -19138,10 +19147,10 @@
         <v>10</v>
       </c>
       <c r="C252" s="1" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D252" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E252" s="1">
         <v>251</v>
@@ -19179,10 +19188,10 @@
         <v>10</v>
       </c>
       <c r="C253" s="1" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D253" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E253" s="1">
         <v>252</v>
@@ -19220,10 +19229,10 @@
         <v>10</v>
       </c>
       <c r="C254" s="1" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D254" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E254" s="1">
         <v>253</v>
@@ -19261,7 +19270,7 @@
         <v>10</v>
       </c>
       <c r="C255" s="1" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D255" s="1" t="s">
         <v>502</v>
@@ -19302,7 +19311,7 @@
         <v>10</v>
       </c>
       <c r="C256" s="1" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D256" s="1" t="s">
         <v>503</v>
@@ -19343,10 +19352,10 @@
         <v>10</v>
       </c>
       <c r="C257" s="1" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="D257" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E257" s="1">
         <v>256</v>
@@ -19384,10 +19393,10 @@
         <v>10</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="D258" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E258" s="1">
         <v>257</v>
@@ -19422,13 +19431,13 @@
         <v>486</v>
       </c>
       <c r="B259" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C259" s="1" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D259" s="1" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="E259" s="1">
         <v>258</v>
@@ -19449,10 +19458,10 @@
         <v>14</v>
       </c>
       <c r="K259" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L259" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M259" s="2" t="s">
         <v>14</v>
@@ -19463,13 +19472,13 @@
         <v>486</v>
       </c>
       <c r="B260" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C260" s="1" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D260" s="1" t="s">
-        <v>495</v>
+        <v>508</v>
       </c>
       <c r="E260" s="1">
         <v>259</v>
@@ -19490,10 +19499,10 @@
         <v>14</v>
       </c>
       <c r="K260" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L260" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M260" s="2" t="s">
         <v>14</v>
@@ -19507,10 +19516,10 @@
         <v>11</v>
       </c>
       <c r="C261" s="1" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="D261" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E261" s="1">
         <v>260</v>
@@ -19548,10 +19557,10 @@
         <v>11</v>
       </c>
       <c r="C262" s="1" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="D262" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E262" s="1">
         <v>261</v>
@@ -19589,10 +19598,10 @@
         <v>11</v>
       </c>
       <c r="C263" s="1" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="D263" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E263" s="1">
         <v>262</v>
@@ -19630,10 +19639,10 @@
         <v>11</v>
       </c>
       <c r="C264" s="1" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="D264" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E264" s="1">
         <v>263</v>
@@ -19671,10 +19680,10 @@
         <v>11</v>
       </c>
       <c r="C265" s="1" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="D265" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E265" s="1">
         <v>264</v>
@@ -19709,13 +19718,13 @@
         <v>486</v>
       </c>
       <c r="B266" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C266" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D266" s="1" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="E266" s="1">
         <v>265</v>
@@ -19750,13 +19759,13 @@
         <v>486</v>
       </c>
       <c r="B267" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C267" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D267" s="1" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="E267" s="1">
         <v>266</v>
@@ -19794,10 +19803,10 @@
         <v>12</v>
       </c>
       <c r="C268" s="1" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D268" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E268" s="1">
         <v>267</v>
@@ -19835,10 +19844,10 @@
         <v>12</v>
       </c>
       <c r="C269" s="1" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D269" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E269" s="1">
         <v>268</v>
@@ -19876,10 +19885,10 @@
         <v>12</v>
       </c>
       <c r="C270" s="1" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D270" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E270" s="1">
         <v>269</v>
@@ -19917,10 +19926,10 @@
         <v>12</v>
       </c>
       <c r="C271" s="1" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D271" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E271" s="1">
         <v>270</v>
@@ -19958,10 +19967,10 @@
         <v>12</v>
       </c>
       <c r="C272" s="1" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D272" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E272" s="1">
         <v>271</v>
@@ -19996,13 +20005,13 @@
         <v>486</v>
       </c>
       <c r="B273" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C273" s="1" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D273" s="1" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="E273" s="1">
         <v>272</v>
@@ -20037,13 +20046,13 @@
         <v>486</v>
       </c>
       <c r="B274" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C274" s="1" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D274" s="1" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="E274" s="1">
         <v>273</v>
@@ -20081,10 +20090,10 @@
         <v>13</v>
       </c>
       <c r="C275" s="1" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="D275" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E275" s="1">
         <v>274</v>
@@ -20122,10 +20131,10 @@
         <v>13</v>
       </c>
       <c r="C276" s="1" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="D276" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E276" s="1">
         <v>275</v>
@@ -20163,10 +20172,10 @@
         <v>13</v>
       </c>
       <c r="C277" s="1" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="D277" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E277" s="1">
         <v>276</v>
@@ -20204,10 +20213,10 @@
         <v>13</v>
       </c>
       <c r="C278" s="1" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="D278" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E278" s="1">
         <v>277</v>
@@ -20245,10 +20254,10 @@
         <v>13</v>
       </c>
       <c r="C279" s="1" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="D279" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E279" s="1">
         <v>278</v>
@@ -20283,13 +20292,13 @@
         <v>486</v>
       </c>
       <c r="B280" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C280" s="1" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D280" s="1" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="E280" s="1">
         <v>279</v>
@@ -20324,13 +20333,13 @@
         <v>486</v>
       </c>
       <c r="B281" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C281" s="1" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D281" s="1" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="E281" s="1">
         <v>280</v>
@@ -20368,10 +20377,10 @@
         <v>14</v>
       </c>
       <c r="C282" s="1" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="D282" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E282" s="1">
         <v>281</v>
@@ -20409,10 +20418,10 @@
         <v>14</v>
       </c>
       <c r="C283" s="1" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="D283" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E283" s="1">
         <v>282</v>
@@ -20450,10 +20459,10 @@
         <v>14</v>
       </c>
       <c r="C284" s="1" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="D284" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E284" s="1">
         <v>283</v>
@@ -20491,10 +20500,10 @@
         <v>14</v>
       </c>
       <c r="C285" s="1" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="D285" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E285" s="1">
         <v>284</v>
@@ -20532,10 +20541,10 @@
         <v>14</v>
       </c>
       <c r="C286" s="1" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="D286" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E286" s="1">
         <v>285</v>
@@ -20570,13 +20579,13 @@
         <v>486</v>
       </c>
       <c r="B287" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C287" s="1" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D287" s="1" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="E287" s="1">
         <v>286</v>
@@ -20611,13 +20620,13 @@
         <v>486</v>
       </c>
       <c r="B288" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C288" s="1" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D288" s="1" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="E288" s="1">
         <v>287</v>
@@ -20655,10 +20664,10 @@
         <v>15</v>
       </c>
       <c r="C289" s="1" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="D289" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E289" s="1">
         <v>288</v>
@@ -20696,10 +20705,10 @@
         <v>15</v>
       </c>
       <c r="C290" s="1" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="D290" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E290" s="1">
         <v>289</v>
@@ -20737,10 +20746,10 @@
         <v>15</v>
       </c>
       <c r="C291" s="1" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="D291" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E291" s="1">
         <v>290</v>
@@ -20778,10 +20787,10 @@
         <v>15</v>
       </c>
       <c r="C292" s="1" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="D292" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E292" s="1">
         <v>291</v>
@@ -20819,10 +20828,10 @@
         <v>15</v>
       </c>
       <c r="C293" s="1" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="D293" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E293" s="1">
         <v>292</v>
@@ -20857,13 +20866,13 @@
         <v>486</v>
       </c>
       <c r="B294" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C294" s="1" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="D294" s="1" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="E294" s="1">
         <v>293</v>
@@ -20898,13 +20907,13 @@
         <v>486</v>
       </c>
       <c r="B295" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C295" s="1" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="D295" s="1" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="E295" s="1">
         <v>294</v>
@@ -20942,10 +20951,10 @@
         <v>16</v>
       </c>
       <c r="C296" s="1" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="D296" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E296" s="1">
         <v>295</v>
@@ -20983,10 +20992,10 @@
         <v>16</v>
       </c>
       <c r="C297" s="1" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="D297" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E297" s="1">
         <v>296</v>
@@ -21024,10 +21033,10 @@
         <v>16</v>
       </c>
       <c r="C298" s="1" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="D298" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E298" s="1">
         <v>297</v>
@@ -21065,10 +21074,10 @@
         <v>16</v>
       </c>
       <c r="C299" s="1" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="D299" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E299" s="1">
         <v>298</v>
@@ -21106,10 +21115,10 @@
         <v>16</v>
       </c>
       <c r="C300" s="1" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="D300" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E300" s="1">
         <v>299</v>
@@ -21141,16 +21150,16 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="s">
-        <v>522</v>
+        <v>486</v>
       </c>
       <c r="B301" s="1">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C301" s="1" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="D301" s="1" t="s">
-        <v>524</v>
+        <v>502</v>
       </c>
       <c r="E301" s="1">
         <v>300</v>
@@ -21174,24 +21183,24 @@
         <v>14</v>
       </c>
       <c r="L301" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M301" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="s">
-        <v>522</v>
+        <v>486</v>
       </c>
       <c r="B302" s="1">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C302" s="1" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="D302" s="1" t="s">
-        <v>525</v>
+        <v>503</v>
       </c>
       <c r="E302" s="1">
         <v>301</v>
@@ -21215,24 +21224,24 @@
         <v>14</v>
       </c>
       <c r="L302" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M302" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B303" s="1">
         <v>1</v>
       </c>
       <c r="C303" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D303" s="1" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E303" s="1">
         <v>302</v>
@@ -21264,16 +21273,16 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B304" s="1">
         <v>1</v>
       </c>
       <c r="C304" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D304" s="1" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E304" s="1">
         <v>303</v>
@@ -21305,16 +21314,16 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B305" s="1">
         <v>1</v>
       </c>
       <c r="C305" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D305" s="1" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E305" s="1">
         <v>304</v>
@@ -21346,16 +21355,16 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B306" s="1">
         <v>1</v>
       </c>
       <c r="C306" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D306" s="1" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E306" s="1">
         <v>305</v>
@@ -21387,16 +21396,16 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B307" s="1">
         <v>1</v>
       </c>
       <c r="C307" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D307" s="1" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E307" s="1">
         <v>306</v>
@@ -21428,16 +21437,16 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B308" s="1">
         <v>1</v>
       </c>
       <c r="C308" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D308" s="1" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E308" s="1">
         <v>307</v>
@@ -21469,16 +21478,16 @@
     </row>
     <row r="309">
       <c r="A309" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B309" s="1">
         <v>1</v>
       </c>
       <c r="C309" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D309" s="1" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E309" s="1">
         <v>308</v>
@@ -21510,16 +21519,16 @@
     </row>
     <row r="310">
       <c r="A310" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B310" s="1">
         <v>1</v>
       </c>
       <c r="C310" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D310" s="1" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E310" s="1">
         <v>309</v>
@@ -21551,16 +21560,16 @@
     </row>
     <row r="311">
       <c r="A311" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B311" s="1">
         <v>1</v>
       </c>
       <c r="C311" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D311" s="1" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E311" s="1">
         <v>310</v>
@@ -21592,16 +21601,16 @@
     </row>
     <row r="312">
       <c r="A312" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B312" s="1">
         <v>1</v>
       </c>
       <c r="C312" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D312" s="1" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E312" s="1">
         <v>311</v>
@@ -21633,16 +21642,16 @@
     </row>
     <row r="313">
       <c r="A313" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B313" s="1">
         <v>1</v>
       </c>
       <c r="C313" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D313" s="1" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="E313" s="1">
         <v>312</v>
@@ -21674,16 +21683,16 @@
     </row>
     <row r="314">
       <c r="A314" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B314" s="1">
         <v>1</v>
       </c>
       <c r="C314" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D314" s="1" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E314" s="1">
         <v>313</v>
@@ -21715,16 +21724,16 @@
     </row>
     <row r="315">
       <c r="A315" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B315" s="1">
         <v>1</v>
       </c>
       <c r="C315" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D315" s="1" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="E315" s="1">
         <v>314</v>
@@ -21756,16 +21765,16 @@
     </row>
     <row r="316">
       <c r="A316" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B316" s="1">
         <v>1</v>
       </c>
       <c r="C316" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D316" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="E316" s="1">
         <v>315</v>
@@ -21797,16 +21806,16 @@
     </row>
     <row r="317">
       <c r="A317" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B317" s="1">
         <v>1</v>
       </c>
       <c r="C317" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D317" s="1" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="E317" s="1">
         <v>316</v>
@@ -21838,16 +21847,16 @@
     </row>
     <row r="318">
       <c r="A318" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B318" s="1">
         <v>1</v>
       </c>
       <c r="C318" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D318" s="1" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E318" s="1">
         <v>317</v>
@@ -21874,6 +21883,88 @@
         <v>14</v>
       </c>
       <c r="M318" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="B319" s="1">
+        <v>1</v>
+      </c>
+      <c r="C319" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="D319" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="E319" s="1">
+        <v>318</v>
+      </c>
+      <c r="F319" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G319" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H319" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I319" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J319" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K319" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L319" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M319" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="B320" s="1">
+        <v>1</v>
+      </c>
+      <c r="C320" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="D320" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="E320" s="1">
+        <v>319</v>
+      </c>
+      <c r="F320" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G320" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H320" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I320" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J320" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K320" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L320" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M320" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -21894,28 +21985,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>174</v>
@@ -21923,16 +22014,16 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E2" s="1">
         <v>1</v>
@@ -21946,16 +22037,16 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E3" s="1">
         <v>2</v>
@@ -21964,7 +22055,7 @@
         <v>15</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H3" s="1">
         <v>8</v>
@@ -21975,16 +22066,16 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E4" s="1">
         <v>3</v>
@@ -21993,7 +22084,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H4" s="1">
         <v>7</v>
@@ -22004,16 +22095,16 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E5" s="1">
         <v>4</v>
@@ -22022,7 +22113,7 @@
         <v>15</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H5" s="1">
         <v>11</v>
@@ -22033,16 +22124,16 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E6" s="1">
         <v>5</v>
@@ -22056,16 +22147,16 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E7" s="1">
         <v>6</v>
@@ -22074,7 +22165,7 @@
         <v>15</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H7" s="1">
         <v>9</v>
@@ -22085,16 +22176,16 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E8" s="1">
         <v>7</v>
@@ -22108,16 +22199,16 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E9" s="1">
         <v>8</v>
@@ -22126,7 +22217,7 @@
         <v>15</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H9" s="1">
         <v>17</v>
@@ -22137,16 +22228,16 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>569</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>570</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>566</v>
       </c>
       <c r="E10" s="1">
         <v>9</v>
@@ -22155,7 +22246,7 @@
         <v>15</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H10" s="1">
         <v>16</v>
@@ -22166,16 +22257,16 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E11" s="1">
         <v>10</v>
@@ -22184,7 +22275,7 @@
         <v>15</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>15</v>
@@ -22192,10 +22283,10 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>14</v>
@@ -22204,7 +22295,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H12" s="1">
         <v>1</v>
@@ -22212,10 +22303,10 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>14</v>
@@ -22224,7 +22315,7 @@
         <v>15</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H13" s="1">
         <v>2</v>
@@ -22235,10 +22326,10 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>14</v>
@@ -22247,7 +22338,7 @@
         <v>15</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H14" s="1">
         <v>3</v>
@@ -22258,10 +22349,10 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>14</v>
@@ -22270,7 +22361,7 @@
         <v>15</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H15" s="1">
         <v>4</v>
@@ -22281,10 +22372,10 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>14</v>
@@ -22293,7 +22384,7 @@
         <v>15</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H16" s="1">
         <v>5</v>
@@ -22304,10 +22395,10 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>14</v>
@@ -22316,7 +22407,7 @@
         <v>15</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H17" s="1">
         <v>6</v>
@@ -22327,10 +22418,10 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>14</v>
@@ -22339,7 +22430,7 @@
         <v>15</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H18" s="1">
         <v>10</v>
@@ -22350,10 +22441,10 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>14</v>
@@ -22362,7 +22453,7 @@
         <v>15</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="H19" s="1">
         <v>12</v>
@@ -22373,10 +22464,10 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>14</v>
@@ -22385,7 +22476,7 @@
         <v>15</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H20" s="1">
         <v>13</v>
@@ -22396,10 +22487,10 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>14</v>
@@ -22408,7 +22499,7 @@
         <v>15</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H21" s="1">
         <v>14</v>
@@ -22419,10 +22510,10 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>14</v>
@@ -22431,7 +22522,7 @@
         <v>15</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H22" s="1">
         <v>15</v>
@@ -22442,10 +22533,10 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>14</v>
@@ -22454,7 +22545,7 @@
         <v>15</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H23" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
Fix cancelled orders, packing cutoff, stock movement voiding
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -7404,6 +7404,32 @@
         <v>15</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="1">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>166</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="D64" s="1">
+        <v>63</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="G64" s="4">
+        <v>78.480000000000004</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -7979,6 +8005,14 @@
     <row r="72">
       <c r="B72" s="3" t="s">
         <v>259</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>166</v>
+      </c>
+      <c r="B73" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Hot fix linen inventory setup items
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="8"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -280,7 +280,7 @@
     <t>Disposable Gloves - L</t>
   </si>
   <si>
-    <t>Cable Tie 6"</t>
+    <t>Cable Tie 8"</t>
   </si>
   <si>
     <t>Magic Sponge</t>
@@ -21794,9 +21794,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s">
-        <v>83</v>
-      </c>
+      <c r="A5"/>
       <c r="B5" s="3" t="s">
         <v>185</v>
       </c>
@@ -22050,6 +22048,9 @@
       </c>
     </row>
     <row r="37">
+      <c r="A37" t="s">
+        <v>83</v>
+      </c>
       <c r="B37" s="3" t="s">
         <v>229</v>
       </c>
@@ -65393,7 +65394,6 @@
       <c r="JR118" s="1"/>
     </row>
     <row r="119">
-      <c r="HM119"/>
       <c r="HN119" s="1"/>
       <c r="HO119" s="1"/>
       <c r="HP119" s="1"/>
@@ -65453,7 +65453,6 @@
       <c r="JR119" s="1"/>
     </row>
     <row r="120">
-      <c r="HM120"/>
       <c r="HN120" s="1"/>
       <c r="HO120" s="1"/>
       <c r="HP120" s="1"/>
@@ -65513,7 +65512,6 @@
       <c r="JR120" s="1"/>
     </row>
     <row r="121">
-      <c r="HM121"/>
       <c r="HN121" s="1"/>
       <c r="HO121" s="1"/>
       <c r="HP121" s="1"/>
@@ -65573,7 +65571,6 @@
       <c r="JR121" s="1"/>
     </row>
     <row r="122">
-      <c r="HM122"/>
       <c r="HN122" s="1"/>
       <c r="HO122" s="1"/>
       <c r="HP122" s="1"/>
@@ -65633,7 +65630,6 @@
       <c r="JR122" s="1"/>
     </row>
     <row r="123">
-      <c r="HM123"/>
       <c r="HN123" s="1"/>
       <c r="HO123" s="1"/>
       <c r="HP123" s="1"/>
@@ -65693,7 +65689,6 @@
       <c r="JR123" s="1"/>
     </row>
     <row r="124">
-      <c r="HM124"/>
       <c r="HN124" s="1"/>
       <c r="HO124" s="1"/>
       <c r="HP124" s="1"/>
@@ -65753,7 +65748,6 @@
       <c r="JR124" s="1"/>
     </row>
     <row r="125">
-      <c r="HM125"/>
       <c r="HN125" s="1"/>
       <c r="HO125" s="1"/>
       <c r="HP125" s="1"/>
@@ -65813,7 +65807,6 @@
       <c r="JR125" s="1"/>
     </row>
     <row r="126">
-      <c r="HM126"/>
       <c r="HN126" s="1"/>
       <c r="HO126" s="1"/>
       <c r="HP126" s="1"/>
@@ -65873,7 +65866,6 @@
       <c r="JR126" s="1"/>
     </row>
     <row r="127">
-      <c r="HM127"/>
       <c r="HN127" s="1"/>
       <c r="HO127" s="1"/>
       <c r="HP127" s="1"/>
@@ -65933,7 +65925,6 @@
       <c r="JR127" s="1"/>
     </row>
     <row r="128">
-      <c r="HM128"/>
       <c r="HN128" s="1"/>
       <c r="HO128" s="1"/>
       <c r="HP128" s="1"/>
@@ -65993,7 +65984,6 @@
       <c r="JR128" s="1"/>
     </row>
     <row r="129">
-      <c r="HM129"/>
       <c r="HN129" s="1"/>
       <c r="HO129" s="1"/>
       <c r="HP129" s="1"/>
@@ -66053,7 +66043,6 @@
       <c r="JR129" s="1"/>
     </row>
     <row r="130">
-      <c r="HM130"/>
       <c r="HN130" s="1"/>
       <c r="HO130" s="1"/>
       <c r="HP130" s="1"/>
@@ -66113,7 +66102,6 @@
       <c r="JR130" s="1"/>
     </row>
     <row r="131">
-      <c r="HM131"/>
       <c r="HN131" s="1"/>
       <c r="HO131" s="1"/>
       <c r="HP131" s="1"/>
@@ -66173,7 +66161,6 @@
       <c r="JR131" s="1"/>
     </row>
     <row r="132">
-      <c r="HM132"/>
       <c r="HN132" s="1"/>
       <c r="HO132" s="1"/>
       <c r="HP132" s="1"/>
@@ -66233,7 +66220,6 @@
       <c r="JR132" s="1"/>
     </row>
     <row r="133">
-      <c r="HM133"/>
       <c r="HN133" s="1"/>
       <c r="HO133" s="1"/>
       <c r="HP133" s="1"/>
@@ -66293,7 +66279,6 @@
       <c r="JR133" s="1"/>
     </row>
     <row r="134">
-      <c r="HM134"/>
       <c r="HN134" s="1"/>
       <c r="HO134" s="1"/>
       <c r="HP134" s="1"/>
@@ -66353,7 +66338,6 @@
       <c r="JR134" s="1"/>
     </row>
     <row r="135">
-      <c r="HM135"/>
       <c r="HN135" s="1"/>
       <c r="HO135" s="1"/>
       <c r="HP135" s="1"/>
@@ -66413,7 +66397,6 @@
       <c r="JR135" s="1"/>
     </row>
     <row r="136">
-      <c r="HM136"/>
       <c r="HN136" s="1"/>
       <c r="HO136" s="1"/>
       <c r="HP136" s="1"/>
@@ -66473,7 +66456,6 @@
       <c r="JR136" s="1"/>
     </row>
     <row r="137">
-      <c r="HM137"/>
       <c r="HN137" s="1"/>
       <c r="HO137" s="1"/>
       <c r="HP137" s="1"/>
@@ -66533,7 +66515,6 @@
       <c r="JR137" s="1"/>
     </row>
     <row r="138">
-      <c r="HM138"/>
       <c r="HN138" s="1"/>
       <c r="HO138" s="1"/>
       <c r="HP138" s="1"/>
@@ -66593,7 +66574,6 @@
       <c r="JR138" s="1"/>
     </row>
     <row r="139">
-      <c r="HM139"/>
       <c r="HN139" s="1"/>
       <c r="HO139" s="1"/>
       <c r="HP139" s="1"/>
@@ -66653,7 +66633,6 @@
       <c r="JR139" s="1"/>
     </row>
     <row r="140">
-      <c r="HM140"/>
       <c r="HN140" s="1"/>
       <c r="HO140" s="1"/>
       <c r="HP140" s="1"/>

</xml_diff>

<commit_message>
hot fix linen inventory items
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="10"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -38099,6 +38099,17 @@
       <c r="FG2" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ2" s="1"/>
+      <c r="GK2" s="1"/>
+      <c r="GL2" s="1"/>
+      <c r="GM2" s="1"/>
+      <c r="GN2" s="1"/>
+      <c r="GO2" s="1"/>
+      <c r="GP2" s="1"/>
+      <c r="GQ2" s="1"/>
+      <c r="GR2" s="1"/>
+      <c r="GS2" s="1"/>
+      <c r="GT2" s="1"/>
       <c r="GU2" s="1" t="s">
         <v>15</v>
       </c>
@@ -38196,6 +38207,17 @@
       <c r="FG3" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ3" s="1"/>
+      <c r="GK3" s="1"/>
+      <c r="GL3" s="1"/>
+      <c r="GM3" s="1"/>
+      <c r="GN3" s="1"/>
+      <c r="GO3" s="1"/>
+      <c r="GP3" s="1"/>
+      <c r="GQ3" s="1"/>
+      <c r="GR3" s="1"/>
+      <c r="GS3" s="1"/>
+      <c r="GT3" s="1"/>
       <c r="GU3" s="1" t="s">
         <v>15</v>
       </c>
@@ -38293,6 +38315,17 @@
       <c r="FG4" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ4" s="1"/>
+      <c r="GK4" s="1"/>
+      <c r="GL4" s="1"/>
+      <c r="GM4" s="1"/>
+      <c r="GN4" s="1"/>
+      <c r="GO4" s="1"/>
+      <c r="GP4" s="1"/>
+      <c r="GQ4" s="1"/>
+      <c r="GR4" s="1"/>
+      <c r="GS4" s="1"/>
+      <c r="GT4" s="1"/>
       <c r="GU4" s="1" t="s">
         <v>15</v>
       </c>
@@ -38390,6 +38423,17 @@
       <c r="FG5" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ5" s="1"/>
+      <c r="GK5" s="1"/>
+      <c r="GL5" s="1"/>
+      <c r="GM5" s="1"/>
+      <c r="GN5" s="1"/>
+      <c r="GO5" s="1"/>
+      <c r="GP5" s="1"/>
+      <c r="GQ5" s="1"/>
+      <c r="GR5" s="1"/>
+      <c r="GS5" s="1"/>
+      <c r="GT5" s="1"/>
       <c r="GU5" s="1" t="s">
         <v>15</v>
       </c>
@@ -38487,6 +38531,17 @@
       <c r="FG6" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ6" s="1"/>
+      <c r="GK6" s="1"/>
+      <c r="GL6" s="1"/>
+      <c r="GM6" s="1"/>
+      <c r="GN6" s="1"/>
+      <c r="GO6" s="1"/>
+      <c r="GP6" s="1"/>
+      <c r="GQ6" s="1"/>
+      <c r="GR6" s="1"/>
+      <c r="GS6" s="1"/>
+      <c r="GT6" s="1"/>
       <c r="GU6" s="1" t="s">
         <v>15</v>
       </c>
@@ -38584,6 +38639,17 @@
       <c r="FG7" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ7" s="1"/>
+      <c r="GK7" s="1"/>
+      <c r="GL7" s="1"/>
+      <c r="GM7" s="1"/>
+      <c r="GN7" s="1"/>
+      <c r="GO7" s="1"/>
+      <c r="GP7" s="1"/>
+      <c r="GQ7" s="1"/>
+      <c r="GR7" s="1"/>
+      <c r="GS7" s="1"/>
+      <c r="GT7" s="1"/>
       <c r="GU7" s="1" t="s">
         <v>15</v>
       </c>
@@ -38678,6 +38744,17 @@
       <c r="FG8" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ8" s="1"/>
+      <c r="GK8" s="1"/>
+      <c r="GL8" s="1"/>
+      <c r="GM8" s="1"/>
+      <c r="GN8" s="1"/>
+      <c r="GO8" s="1"/>
+      <c r="GP8" s="1"/>
+      <c r="GQ8" s="1"/>
+      <c r="GR8" s="1"/>
+      <c r="GS8" s="1"/>
+      <c r="GT8" s="1"/>
       <c r="GU8" s="1" t="s">
         <v>15</v>
       </c>
@@ -38772,6 +38849,17 @@
       <c r="FG9" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ9" s="1"/>
+      <c r="GK9" s="1"/>
+      <c r="GL9" s="1"/>
+      <c r="GM9" s="1"/>
+      <c r="GN9" s="1"/>
+      <c r="GO9" s="1"/>
+      <c r="GP9" s="1"/>
+      <c r="GQ9" s="1"/>
+      <c r="GR9" s="1"/>
+      <c r="GS9" s="1"/>
+      <c r="GT9" s="1"/>
       <c r="GU9" s="1" t="s">
         <v>15</v>
       </c>
@@ -38869,6 +38957,17 @@
       <c r="FG10" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ10" s="1"/>
+      <c r="GK10" s="1"/>
+      <c r="GL10" s="1"/>
+      <c r="GM10" s="1"/>
+      <c r="GN10" s="1"/>
+      <c r="GO10" s="1"/>
+      <c r="GP10" s="1"/>
+      <c r="GQ10" s="1"/>
+      <c r="GR10" s="1"/>
+      <c r="GS10" s="1"/>
+      <c r="GT10" s="1"/>
       <c r="GU10" s="1" t="s">
         <v>15</v>
       </c>
@@ -38966,6 +39065,17 @@
       <c r="FG11" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ11" s="1"/>
+      <c r="GK11" s="1"/>
+      <c r="GL11" s="1"/>
+      <c r="GM11" s="1"/>
+      <c r="GN11" s="1"/>
+      <c r="GO11" s="1"/>
+      <c r="GP11" s="1"/>
+      <c r="GQ11" s="1"/>
+      <c r="GR11" s="1"/>
+      <c r="GS11" s="1"/>
+      <c r="GT11" s="1"/>
       <c r="GU11" s="1" t="s">
         <v>15</v>
       </c>
@@ -39063,6 +39173,17 @@
       <c r="FG12" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ12" s="1"/>
+      <c r="GK12" s="1"/>
+      <c r="GL12" s="1"/>
+      <c r="GM12" s="1"/>
+      <c r="GN12" s="1"/>
+      <c r="GO12" s="1"/>
+      <c r="GP12" s="1"/>
+      <c r="GQ12" s="1"/>
+      <c r="GR12" s="1"/>
+      <c r="GS12" s="1"/>
+      <c r="GT12" s="1"/>
       <c r="GU12" s="1" t="s">
         <v>15</v>
       </c>
@@ -39157,6 +39278,17 @@
       <c r="FG13" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ13" s="1"/>
+      <c r="GK13" s="1"/>
+      <c r="GL13" s="1"/>
+      <c r="GM13" s="1"/>
+      <c r="GN13" s="1"/>
+      <c r="GO13" s="1"/>
+      <c r="GP13" s="1"/>
+      <c r="GQ13" s="1"/>
+      <c r="GR13" s="1"/>
+      <c r="GS13" s="1"/>
+      <c r="GT13" s="1"/>
       <c r="GU13" s="1" t="s">
         <v>15</v>
       </c>
@@ -39251,6 +39383,17 @@
       <c r="FG14" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ14" s="1"/>
+      <c r="GK14" s="1"/>
+      <c r="GL14" s="1"/>
+      <c r="GM14" s="1"/>
+      <c r="GN14" s="1"/>
+      <c r="GO14" s="1"/>
+      <c r="GP14" s="1"/>
+      <c r="GQ14" s="1"/>
+      <c r="GR14" s="1"/>
+      <c r="GS14" s="1"/>
+      <c r="GT14" s="1"/>
       <c r="GU14" s="1" t="s">
         <v>15</v>
       </c>
@@ -39351,6 +39494,17 @@
       <c r="FG15" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ15" s="1"/>
+      <c r="GK15" s="1"/>
+      <c r="GL15" s="1"/>
+      <c r="GM15" s="1"/>
+      <c r="GN15" s="1"/>
+      <c r="GO15" s="1"/>
+      <c r="GP15" s="1"/>
+      <c r="GQ15" s="1"/>
+      <c r="GR15" s="1"/>
+      <c r="GS15" s="1"/>
+      <c r="GT15" s="1"/>
       <c r="GU15" s="1" t="s">
         <v>15</v>
       </c>
@@ -39451,6 +39605,17 @@
       <c r="FG16" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ16" s="1"/>
+      <c r="GK16" s="1"/>
+      <c r="GL16" s="1"/>
+      <c r="GM16" s="1"/>
+      <c r="GN16" s="1"/>
+      <c r="GO16" s="1"/>
+      <c r="GP16" s="1"/>
+      <c r="GQ16" s="1"/>
+      <c r="GR16" s="1"/>
+      <c r="GS16" s="1"/>
+      <c r="GT16" s="1"/>
       <c r="GU16" s="1" t="s">
         <v>15</v>
       </c>
@@ -39551,6 +39716,17 @@
       <c r="FG17" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ17" s="1"/>
+      <c r="GK17" s="1"/>
+      <c r="GL17" s="1"/>
+      <c r="GM17" s="1"/>
+      <c r="GN17" s="1"/>
+      <c r="GO17" s="1"/>
+      <c r="GP17" s="1"/>
+      <c r="GQ17" s="1"/>
+      <c r="GR17" s="1"/>
+      <c r="GS17" s="1"/>
+      <c r="GT17" s="1"/>
       <c r="GU17" s="1" t="s">
         <v>15</v>
       </c>
@@ -39840,6 +40016,39 @@
       <c r="GI18" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GK18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GL18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GM18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GN18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GO18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GP18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GQ18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GR18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GS18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GT18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="GU18" s="1" t="s">
         <v>15</v>
       </c>
@@ -39873,7 +40082,9 @@
         <v>15</v>
       </c>
       <c r="HO18" s="1"/>
-      <c r="HP18" s="1"/>
+      <c r="HP18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HQ18" s="1"/>
       <c r="HR18" s="1" t="s">
         <v>15</v>
@@ -39890,7 +40101,9 @@
         <v>15</v>
       </c>
       <c r="HX18" s="1"/>
-      <c r="HY18" s="1"/>
+      <c r="HY18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HZ18" s="1"/>
       <c r="IA18" s="1" t="s">
         <v>15</v>
@@ -39900,55 +40113,73 @@
         <v>15</v>
       </c>
       <c r="ID18" s="1"/>
-      <c r="IE18" s="1"/>
+      <c r="IE18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IF18" s="1"/>
       <c r="IG18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IH18" s="1"/>
-      <c r="II18" s="1"/>
+      <c r="II18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IJ18" s="1"/>
       <c r="IK18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IL18" s="1"/>
-      <c r="IM18" s="1"/>
+      <c r="IM18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IN18" s="1"/>
       <c r="IO18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IP18" s="1"/>
-      <c r="IQ18" s="1"/>
+      <c r="IQ18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IR18" s="1"/>
       <c r="IS18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IT18" s="1"/>
-      <c r="IU18" s="1"/>
+      <c r="IU18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IV18" s="1"/>
       <c r="IW18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IX18" s="1"/>
-      <c r="IY18" s="1"/>
+      <c r="IY18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IZ18" s="1"/>
       <c r="JA18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JB18" s="1"/>
-      <c r="JC18" s="1"/>
+      <c r="JC18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JD18" s="1"/>
       <c r="JE18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JF18" s="1"/>
-      <c r="JG18" s="1"/>
+      <c r="JG18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JH18" s="1"/>
       <c r="JI18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JJ18" s="1"/>
-      <c r="JK18" s="1"/>
+      <c r="JK18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JL18" s="1"/>
       <c r="JM18" s="1" t="s">
         <v>15</v>
@@ -40806,6 +41037,9 @@
       <c r="BZ21" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CA21" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CD21" s="1" t="s">
         <v>15</v>
       </c>
@@ -41947,39 +42181,17 @@
       <c r="GI23" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="GJ23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GK23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GL23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GM23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GN23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GO23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GP23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GQ23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GR23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GS23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GT23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="GJ23" s="1"/>
+      <c r="GK23" s="1"/>
+      <c r="GL23" s="1"/>
+      <c r="GM23" s="1"/>
+      <c r="GN23" s="1"/>
+      <c r="GO23" s="1"/>
+      <c r="GP23" s="1"/>
+      <c r="GQ23" s="1"/>
+      <c r="GR23" s="1"/>
+      <c r="GS23" s="1"/>
+      <c r="GT23" s="1"/>
       <c r="GU23" s="1" t="s">
         <v>15</v>
       </c>
@@ -42030,9 +42242,7 @@
         <v>15</v>
       </c>
       <c r="HO23" s="1"/>
-      <c r="HP23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="HP23" s="1"/>
       <c r="HQ23" s="1"/>
       <c r="HR23" s="1" t="s">
         <v>15</v>
@@ -42049,9 +42259,7 @@
         <v>15</v>
       </c>
       <c r="HX23" s="1"/>
-      <c r="HY23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="HY23" s="1"/>
       <c r="HZ23" s="1"/>
       <c r="IA23" s="1" t="s">
         <v>15</v>
@@ -42061,73 +42269,55 @@
         <v>15</v>
       </c>
       <c r="ID23" s="1"/>
-      <c r="IE23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IE23" s="1"/>
       <c r="IF23" s="1"/>
       <c r="IG23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IH23" s="1"/>
-      <c r="II23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="II23" s="1"/>
       <c r="IJ23" s="1"/>
       <c r="IK23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IL23" s="1"/>
-      <c r="IM23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IM23" s="1"/>
       <c r="IN23" s="1"/>
       <c r="IO23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IP23" s="1"/>
-      <c r="IQ23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IQ23" s="1"/>
       <c r="IR23" s="1"/>
       <c r="IS23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IT23" s="1"/>
-      <c r="IU23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IU23" s="1"/>
       <c r="IV23" s="1"/>
       <c r="IW23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IX23" s="1"/>
-      <c r="IY23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IY23" s="1"/>
       <c r="IZ23" s="1"/>
       <c r="JA23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JB23" s="1"/>
-      <c r="JC23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="JC23" s="1"/>
       <c r="JD23" s="1"/>
       <c r="JE23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JF23" s="1"/>
-      <c r="JG23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="JG23" s="1"/>
       <c r="JH23" s="1"/>
       <c r="JI23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JJ23" s="1"/>
-      <c r="JK23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="JK23" s="1"/>
       <c r="JL23" s="1"/>
       <c r="JM23" s="1" t="s">
         <v>15</v>
@@ -42235,6 +42425,17 @@
       <c r="FN24" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ24" s="1"/>
+      <c r="GK24" s="1"/>
+      <c r="GL24" s="1"/>
+      <c r="GM24" s="1"/>
+      <c r="GN24" s="1"/>
+      <c r="GO24" s="1"/>
+      <c r="GP24" s="1"/>
+      <c r="GQ24" s="1"/>
+      <c r="GR24" s="1"/>
+      <c r="GS24" s="1"/>
+      <c r="GT24" s="1"/>
       <c r="GU24" s="1" t="s">
         <v>15</v>
       </c>
@@ -42341,6 +42542,17 @@
       <c r="FM25" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ25" s="1"/>
+      <c r="GK25" s="1"/>
+      <c r="GL25" s="1"/>
+      <c r="GM25" s="1"/>
+      <c r="GN25" s="1"/>
+      <c r="GO25" s="1"/>
+      <c r="GP25" s="1"/>
+      <c r="GQ25" s="1"/>
+      <c r="GR25" s="1"/>
+      <c r="GS25" s="1"/>
+      <c r="GT25" s="1"/>
       <c r="GU25" s="1" t="s">
         <v>15</v>
       </c>
@@ -42438,6 +42650,17 @@
       <c r="FG26" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ26" s="1"/>
+      <c r="GK26" s="1"/>
+      <c r="GL26" s="1"/>
+      <c r="GM26" s="1"/>
+      <c r="GN26" s="1"/>
+      <c r="GO26" s="1"/>
+      <c r="GP26" s="1"/>
+      <c r="GQ26" s="1"/>
+      <c r="GR26" s="1"/>
+      <c r="GS26" s="1"/>
+      <c r="GT26" s="1"/>
       <c r="GU26" s="1" t="s">
         <v>15</v>
       </c>
@@ -42535,6 +42758,17 @@
       <c r="FG27" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ27" s="1"/>
+      <c r="GK27" s="1"/>
+      <c r="GL27" s="1"/>
+      <c r="GM27" s="1"/>
+      <c r="GN27" s="1"/>
+      <c r="GO27" s="1"/>
+      <c r="GP27" s="1"/>
+      <c r="GQ27" s="1"/>
+      <c r="GR27" s="1"/>
+      <c r="GS27" s="1"/>
+      <c r="GT27" s="1"/>
       <c r="GU27" s="1" t="s">
         <v>15</v>
       </c>
@@ -42632,6 +42866,17 @@
       <c r="FG28" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ28" s="1"/>
+      <c r="GK28" s="1"/>
+      <c r="GL28" s="1"/>
+      <c r="GM28" s="1"/>
+      <c r="GN28" s="1"/>
+      <c r="GO28" s="1"/>
+      <c r="GP28" s="1"/>
+      <c r="GQ28" s="1"/>
+      <c r="GR28" s="1"/>
+      <c r="GS28" s="1"/>
+      <c r="GT28" s="1"/>
       <c r="GU28" s="1" t="s">
         <v>15</v>
       </c>
@@ -42741,6 +42986,17 @@
       <c r="FN29" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ29" s="1"/>
+      <c r="GK29" s="1"/>
+      <c r="GL29" s="1"/>
+      <c r="GM29" s="1"/>
+      <c r="GN29" s="1"/>
+      <c r="GO29" s="1"/>
+      <c r="GP29" s="1"/>
+      <c r="GQ29" s="1"/>
+      <c r="GR29" s="1"/>
+      <c r="GS29" s="1"/>
+      <c r="GT29" s="1"/>
       <c r="GU29" s="1" t="s">
         <v>15</v>
       </c>
@@ -42838,6 +43094,17 @@
       <c r="FG30" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ30" s="1"/>
+      <c r="GK30" s="1"/>
+      <c r="GL30" s="1"/>
+      <c r="GM30" s="1"/>
+      <c r="GN30" s="1"/>
+      <c r="GO30" s="1"/>
+      <c r="GP30" s="1"/>
+      <c r="GQ30" s="1"/>
+      <c r="GR30" s="1"/>
+      <c r="GS30" s="1"/>
+      <c r="GT30" s="1"/>
       <c r="GU30" s="1" t="s">
         <v>15</v>
       </c>
@@ -42932,6 +43199,17 @@
       <c r="FG31" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ31" s="1"/>
+      <c r="GK31" s="1"/>
+      <c r="GL31" s="1"/>
+      <c r="GM31" s="1"/>
+      <c r="GN31" s="1"/>
+      <c r="GO31" s="1"/>
+      <c r="GP31" s="1"/>
+      <c r="GQ31" s="1"/>
+      <c r="GR31" s="1"/>
+      <c r="GS31" s="1"/>
+      <c r="GT31" s="1"/>
       <c r="GU31" s="1" t="s">
         <v>15</v>
       </c>
@@ -43029,6 +43307,17 @@
       <c r="FG32" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ32" s="1"/>
+      <c r="GK32" s="1"/>
+      <c r="GL32" s="1"/>
+      <c r="GM32" s="1"/>
+      <c r="GN32" s="1"/>
+      <c r="GO32" s="1"/>
+      <c r="GP32" s="1"/>
+      <c r="GQ32" s="1"/>
+      <c r="GR32" s="1"/>
+      <c r="GS32" s="1"/>
+      <c r="GT32" s="1"/>
       <c r="GU32" s="1" t="s">
         <v>15</v>
       </c>
@@ -43123,6 +43412,17 @@
       <c r="FG33" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ33" s="1"/>
+      <c r="GK33" s="1"/>
+      <c r="GL33" s="1"/>
+      <c r="GM33" s="1"/>
+      <c r="GN33" s="1"/>
+      <c r="GO33" s="1"/>
+      <c r="GP33" s="1"/>
+      <c r="GQ33" s="1"/>
+      <c r="GR33" s="1"/>
+      <c r="GS33" s="1"/>
+      <c r="GT33" s="1"/>
       <c r="GU33" s="1" t="s">
         <v>15</v>
       </c>
@@ -43220,6 +43520,17 @@
       <c r="FG34" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ34" s="1"/>
+      <c r="GK34" s="1"/>
+      <c r="GL34" s="1"/>
+      <c r="GM34" s="1"/>
+      <c r="GN34" s="1"/>
+      <c r="GO34" s="1"/>
+      <c r="GP34" s="1"/>
+      <c r="GQ34" s="1"/>
+      <c r="GR34" s="1"/>
+      <c r="GS34" s="1"/>
+      <c r="GT34" s="1"/>
       <c r="GU34" s="1" t="s">
         <v>15</v>
       </c>
@@ -43317,6 +43628,17 @@
       <c r="FG35" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ35" s="1"/>
+      <c r="GK35" s="1"/>
+      <c r="GL35" s="1"/>
+      <c r="GM35" s="1"/>
+      <c r="GN35" s="1"/>
+      <c r="GO35" s="1"/>
+      <c r="GP35" s="1"/>
+      <c r="GQ35" s="1"/>
+      <c r="GR35" s="1"/>
+      <c r="GS35" s="1"/>
+      <c r="GT35" s="1"/>
       <c r="GU35" s="1" t="s">
         <v>15</v>
       </c>
@@ -43414,6 +43736,17 @@
       <c r="FG36" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ36" s="1"/>
+      <c r="GK36" s="1"/>
+      <c r="GL36" s="1"/>
+      <c r="GM36" s="1"/>
+      <c r="GN36" s="1"/>
+      <c r="GO36" s="1"/>
+      <c r="GP36" s="1"/>
+      <c r="GQ36" s="1"/>
+      <c r="GR36" s="1"/>
+      <c r="GS36" s="1"/>
+      <c r="GT36" s="1"/>
       <c r="GU36" s="1" t="s">
         <v>15</v>
       </c>
@@ -43508,6 +43841,17 @@
       <c r="FG37" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ37" s="1"/>
+      <c r="GK37" s="1"/>
+      <c r="GL37" s="1"/>
+      <c r="GM37" s="1"/>
+      <c r="GN37" s="1"/>
+      <c r="GO37" s="1"/>
+      <c r="GP37" s="1"/>
+      <c r="GQ37" s="1"/>
+      <c r="GR37" s="1"/>
+      <c r="GS37" s="1"/>
+      <c r="GT37" s="1"/>
       <c r="GU37" s="1" t="s">
         <v>15</v>
       </c>
@@ -43602,6 +43946,17 @@
       <c r="FG38" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ38" s="1"/>
+      <c r="GK38" s="1"/>
+      <c r="GL38" s="1"/>
+      <c r="GM38" s="1"/>
+      <c r="GN38" s="1"/>
+      <c r="GO38" s="1"/>
+      <c r="GP38" s="1"/>
+      <c r="GQ38" s="1"/>
+      <c r="GR38" s="1"/>
+      <c r="GS38" s="1"/>
+      <c r="GT38" s="1"/>
       <c r="GU38" s="1" t="s">
         <v>15</v>
       </c>
@@ -43696,6 +44051,17 @@
       <c r="FG39" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ39" s="1"/>
+      <c r="GK39" s="1"/>
+      <c r="GL39" s="1"/>
+      <c r="GM39" s="1"/>
+      <c r="GN39" s="1"/>
+      <c r="GO39" s="1"/>
+      <c r="GP39" s="1"/>
+      <c r="GQ39" s="1"/>
+      <c r="GR39" s="1"/>
+      <c r="GS39" s="1"/>
+      <c r="GT39" s="1"/>
       <c r="GU39" s="1" t="s">
         <v>15</v>
       </c>
@@ -43790,6 +44156,17 @@
       <c r="FG40" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ40" s="1"/>
+      <c r="GK40" s="1"/>
+      <c r="GL40" s="1"/>
+      <c r="GM40" s="1"/>
+      <c r="GN40" s="1"/>
+      <c r="GO40" s="1"/>
+      <c r="GP40" s="1"/>
+      <c r="GQ40" s="1"/>
+      <c r="GR40" s="1"/>
+      <c r="GS40" s="1"/>
+      <c r="GT40" s="1"/>
       <c r="GU40" s="1" t="s">
         <v>15</v>
       </c>
@@ -43884,6 +44261,17 @@
       <c r="FG41" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ41" s="1"/>
+      <c r="GK41" s="1"/>
+      <c r="GL41" s="1"/>
+      <c r="GM41" s="1"/>
+      <c r="GN41" s="1"/>
+      <c r="GO41" s="1"/>
+      <c r="GP41" s="1"/>
+      <c r="GQ41" s="1"/>
+      <c r="GR41" s="1"/>
+      <c r="GS41" s="1"/>
+      <c r="GT41" s="1"/>
       <c r="GU41" s="1" t="s">
         <v>15</v>
       </c>
@@ -44257,6 +44645,17 @@
       <c r="FQ42" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ42" s="1"/>
+      <c r="GK42" s="1"/>
+      <c r="GL42" s="1"/>
+      <c r="GM42" s="1"/>
+      <c r="GN42" s="1"/>
+      <c r="GO42" s="1"/>
+      <c r="GP42" s="1"/>
+      <c r="GQ42" s="1"/>
+      <c r="GR42" s="1"/>
+      <c r="GS42" s="1"/>
+      <c r="GT42" s="1"/>
       <c r="GU42" s="1" t="s">
         <v>15</v>
       </c>
@@ -44742,6 +45141,17 @@
       <c r="FQ43" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ43" s="1"/>
+      <c r="GK43" s="1"/>
+      <c r="GL43" s="1"/>
+      <c r="GM43" s="1"/>
+      <c r="GN43" s="1"/>
+      <c r="GO43" s="1"/>
+      <c r="GP43" s="1"/>
+      <c r="GQ43" s="1"/>
+      <c r="GR43" s="1"/>
+      <c r="GS43" s="1"/>
+      <c r="GT43" s="1"/>
       <c r="GU43" s="1" t="s">
         <v>15</v>
       </c>
@@ -45236,6 +45646,17 @@
       <c r="FQ44" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ44" s="1"/>
+      <c r="GK44" s="1"/>
+      <c r="GL44" s="1"/>
+      <c r="GM44" s="1"/>
+      <c r="GN44" s="1"/>
+      <c r="GO44" s="1"/>
+      <c r="GP44" s="1"/>
+      <c r="GQ44" s="1"/>
+      <c r="GR44" s="1"/>
+      <c r="GS44" s="1"/>
+      <c r="GT44" s="1"/>
       <c r="GU44" s="1" t="s">
         <v>15</v>
       </c>
@@ -45673,6 +46094,17 @@
       <c r="FQ45" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ45" s="1"/>
+      <c r="GK45" s="1"/>
+      <c r="GL45" s="1"/>
+      <c r="GM45" s="1"/>
+      <c r="GN45" s="1"/>
+      <c r="GO45" s="1"/>
+      <c r="GP45" s="1"/>
+      <c r="GQ45" s="1"/>
+      <c r="GR45" s="1"/>
+      <c r="GS45" s="1"/>
+      <c r="GT45" s="1"/>
       <c r="GU45" s="1" t="s">
         <v>15</v>
       </c>
@@ -46672,6 +47104,17 @@
       <c r="FG47" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ47" s="1"/>
+      <c r="GK47" s="1"/>
+      <c r="GL47" s="1"/>
+      <c r="GM47" s="1"/>
+      <c r="GN47" s="1"/>
+      <c r="GO47" s="1"/>
+      <c r="GP47" s="1"/>
+      <c r="GQ47" s="1"/>
+      <c r="GR47" s="1"/>
+      <c r="GS47" s="1"/>
+      <c r="GT47" s="1"/>
       <c r="GU47" s="1" t="s">
         <v>15</v>
       </c>
@@ -47127,6 +47570,17 @@
       <c r="FQ48" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ48" s="1"/>
+      <c r="GK48" s="1"/>
+      <c r="GL48" s="1"/>
+      <c r="GM48" s="1"/>
+      <c r="GN48" s="1"/>
+      <c r="GO48" s="1"/>
+      <c r="GP48" s="1"/>
+      <c r="GQ48" s="1"/>
+      <c r="GR48" s="1"/>
+      <c r="GS48" s="1"/>
+      <c r="GT48" s="1"/>
       <c r="GU48" s="1" t="s">
         <v>15</v>
       </c>
@@ -47612,6 +48066,17 @@
       <c r="FQ49" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ49" s="1"/>
+      <c r="GK49" s="1"/>
+      <c r="GL49" s="1"/>
+      <c r="GM49" s="1"/>
+      <c r="GN49" s="1"/>
+      <c r="GO49" s="1"/>
+      <c r="GP49" s="1"/>
+      <c r="GQ49" s="1"/>
+      <c r="GR49" s="1"/>
+      <c r="GS49" s="1"/>
+      <c r="GT49" s="1"/>
       <c r="GU49" s="1" t="s">
         <v>15</v>
       </c>
@@ -48106,6 +48571,17 @@
       <c r="FQ50" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ50" s="1"/>
+      <c r="GK50" s="1"/>
+      <c r="GL50" s="1"/>
+      <c r="GM50" s="1"/>
+      <c r="GN50" s="1"/>
+      <c r="GO50" s="1"/>
+      <c r="GP50" s="1"/>
+      <c r="GQ50" s="1"/>
+      <c r="GR50" s="1"/>
+      <c r="GS50" s="1"/>
+      <c r="GT50" s="1"/>
       <c r="GU50" s="1" t="s">
         <v>15</v>
       </c>
@@ -48543,6 +49019,17 @@
       <c r="FQ51" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ51" s="1"/>
+      <c r="GK51" s="1"/>
+      <c r="GL51" s="1"/>
+      <c r="GM51" s="1"/>
+      <c r="GN51" s="1"/>
+      <c r="GO51" s="1"/>
+      <c r="GP51" s="1"/>
+      <c r="GQ51" s="1"/>
+      <c r="GR51" s="1"/>
+      <c r="GS51" s="1"/>
+      <c r="GT51" s="1"/>
       <c r="GU51" s="1" t="s">
         <v>15</v>
       </c>
@@ -49542,6 +50029,17 @@
       <c r="FG53" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ53" s="1"/>
+      <c r="GK53" s="1"/>
+      <c r="GL53" s="1"/>
+      <c r="GM53" s="1"/>
+      <c r="GN53" s="1"/>
+      <c r="GO53" s="1"/>
+      <c r="GP53" s="1"/>
+      <c r="GQ53" s="1"/>
+      <c r="GR53" s="1"/>
+      <c r="GS53" s="1"/>
+      <c r="GT53" s="1"/>
       <c r="GU53" s="1" t="s">
         <v>15</v>
       </c>
@@ -50003,6 +50501,17 @@
       <c r="FQ54" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ54" s="1"/>
+      <c r="GK54" s="1"/>
+      <c r="GL54" s="1"/>
+      <c r="GM54" s="1"/>
+      <c r="GN54" s="1"/>
+      <c r="GO54" s="1"/>
+      <c r="GP54" s="1"/>
+      <c r="GQ54" s="1"/>
+      <c r="GR54" s="1"/>
+      <c r="GS54" s="1"/>
+      <c r="GT54" s="1"/>
       <c r="GU54" s="1" t="s">
         <v>15</v>
       </c>
@@ -50488,6 +50997,17 @@
       <c r="FQ55" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ55" s="1"/>
+      <c r="GK55" s="1"/>
+      <c r="GL55" s="1"/>
+      <c r="GM55" s="1"/>
+      <c r="GN55" s="1"/>
+      <c r="GO55" s="1"/>
+      <c r="GP55" s="1"/>
+      <c r="GQ55" s="1"/>
+      <c r="GR55" s="1"/>
+      <c r="GS55" s="1"/>
+      <c r="GT55" s="1"/>
       <c r="GU55" s="1" t="s">
         <v>15</v>
       </c>
@@ -50988,6 +51508,17 @@
       <c r="FQ56" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ56" s="1"/>
+      <c r="GK56" s="1"/>
+      <c r="GL56" s="1"/>
+      <c r="GM56" s="1"/>
+      <c r="GN56" s="1"/>
+      <c r="GO56" s="1"/>
+      <c r="GP56" s="1"/>
+      <c r="GQ56" s="1"/>
+      <c r="GR56" s="1"/>
+      <c r="GS56" s="1"/>
+      <c r="GT56" s="1"/>
       <c r="GU56" s="1" t="s">
         <v>15</v>
       </c>
@@ -51431,6 +51962,17 @@
       <c r="FQ57" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ57" s="1"/>
+      <c r="GK57" s="1"/>
+      <c r="GL57" s="1"/>
+      <c r="GM57" s="1"/>
+      <c r="GN57" s="1"/>
+      <c r="GO57" s="1"/>
+      <c r="GP57" s="1"/>
+      <c r="GQ57" s="1"/>
+      <c r="GR57" s="1"/>
+      <c r="GS57" s="1"/>
+      <c r="GT57" s="1"/>
       <c r="GU57" s="1" t="s">
         <v>15</v>
       </c>
@@ -52436,6 +52978,17 @@
       <c r="FG59" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ59" s="1"/>
+      <c r="GK59" s="1"/>
+      <c r="GL59" s="1"/>
+      <c r="GM59" s="1"/>
+      <c r="GN59" s="1"/>
+      <c r="GO59" s="1"/>
+      <c r="GP59" s="1"/>
+      <c r="GQ59" s="1"/>
+      <c r="GR59" s="1"/>
+      <c r="GS59" s="1"/>
+      <c r="GT59" s="1"/>
       <c r="GU59" s="1" t="s">
         <v>15</v>
       </c>
@@ -52897,6 +53450,17 @@
       <c r="FQ60" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ60" s="1"/>
+      <c r="GK60" s="1"/>
+      <c r="GL60" s="1"/>
+      <c r="GM60" s="1"/>
+      <c r="GN60" s="1"/>
+      <c r="GO60" s="1"/>
+      <c r="GP60" s="1"/>
+      <c r="GQ60" s="1"/>
+      <c r="GR60" s="1"/>
+      <c r="GS60" s="1"/>
+      <c r="GT60" s="1"/>
       <c r="GU60" s="1" t="s">
         <v>15</v>
       </c>
@@ -53382,6 +53946,17 @@
       <c r="FQ61" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ61" s="1"/>
+      <c r="GK61" s="1"/>
+      <c r="GL61" s="1"/>
+      <c r="GM61" s="1"/>
+      <c r="GN61" s="1"/>
+      <c r="GO61" s="1"/>
+      <c r="GP61" s="1"/>
+      <c r="GQ61" s="1"/>
+      <c r="GR61" s="1"/>
+      <c r="GS61" s="1"/>
+      <c r="GT61" s="1"/>
       <c r="GU61" s="1" t="s">
         <v>15</v>
       </c>
@@ -53882,6 +54457,17 @@
       <c r="FQ62" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ62" s="1"/>
+      <c r="GK62" s="1"/>
+      <c r="GL62" s="1"/>
+      <c r="GM62" s="1"/>
+      <c r="GN62" s="1"/>
+      <c r="GO62" s="1"/>
+      <c r="GP62" s="1"/>
+      <c r="GQ62" s="1"/>
+      <c r="GR62" s="1"/>
+      <c r="GS62" s="1"/>
+      <c r="GT62" s="1"/>
       <c r="GU62" s="1" t="s">
         <v>15</v>
       </c>
@@ -54325,6 +54911,17 @@
       <c r="FQ63" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ63" s="1"/>
+      <c r="GK63" s="1"/>
+      <c r="GL63" s="1"/>
+      <c r="GM63" s="1"/>
+      <c r="GN63" s="1"/>
+      <c r="GO63" s="1"/>
+      <c r="GP63" s="1"/>
+      <c r="GQ63" s="1"/>
+      <c r="GR63" s="1"/>
+      <c r="GS63" s="1"/>
+      <c r="GT63" s="1"/>
       <c r="GU63" s="1" t="s">
         <v>15</v>
       </c>
@@ -55330,6 +55927,17 @@
       <c r="FG65" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ65" s="1"/>
+      <c r="GK65" s="1"/>
+      <c r="GL65" s="1"/>
+      <c r="GM65" s="1"/>
+      <c r="GN65" s="1"/>
+      <c r="GO65" s="1"/>
+      <c r="GP65" s="1"/>
+      <c r="GQ65" s="1"/>
+      <c r="GR65" s="1"/>
+      <c r="GS65" s="1"/>
+      <c r="GT65" s="1"/>
       <c r="GU65" s="1" t="s">
         <v>15</v>
       </c>
@@ -55722,6 +56330,17 @@
       <c r="FQ66" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ66" s="1"/>
+      <c r="GK66" s="1"/>
+      <c r="GL66" s="1"/>
+      <c r="GM66" s="1"/>
+      <c r="GN66" s="1"/>
+      <c r="GO66" s="1"/>
+      <c r="GP66" s="1"/>
+      <c r="GQ66" s="1"/>
+      <c r="GR66" s="1"/>
+      <c r="GS66" s="1"/>
+      <c r="GT66" s="1"/>
       <c r="GU66" s="1" t="s">
         <v>15</v>
       </c>
@@ -56670,6 +57289,17 @@
       <c r="FQ68" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ68" s="1"/>
+      <c r="GK68" s="1"/>
+      <c r="GL68" s="1"/>
+      <c r="GM68" s="1"/>
+      <c r="GN68" s="1"/>
+      <c r="GO68" s="1"/>
+      <c r="GP68" s="1"/>
+      <c r="GQ68" s="1"/>
+      <c r="GR68" s="1"/>
+      <c r="GS68" s="1"/>
+      <c r="GT68" s="1"/>
       <c r="GU68" s="1" t="s">
         <v>15</v>
       </c>
@@ -57134,6 +57764,17 @@
       <c r="FQ69" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ69" s="1"/>
+      <c r="GK69" s="1"/>
+      <c r="GL69" s="1"/>
+      <c r="GM69" s="1"/>
+      <c r="GN69" s="1"/>
+      <c r="GO69" s="1"/>
+      <c r="GP69" s="1"/>
+      <c r="GQ69" s="1"/>
+      <c r="GR69" s="1"/>
+      <c r="GS69" s="1"/>
+      <c r="GT69" s="1"/>
       <c r="GU69" s="1" t="s">
         <v>15</v>
       </c>
@@ -57590,6 +58231,17 @@
       <c r="FQ70" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ70" s="1"/>
+      <c r="GK70" s="1"/>
+      <c r="GL70" s="1"/>
+      <c r="GM70" s="1"/>
+      <c r="GN70" s="1"/>
+      <c r="GO70" s="1"/>
+      <c r="GP70" s="1"/>
+      <c r="GQ70" s="1"/>
+      <c r="GR70" s="1"/>
+      <c r="GS70" s="1"/>
+      <c r="GT70" s="1"/>
       <c r="GU70" s="1" t="s">
         <v>15</v>
       </c>
@@ -58049,6 +58701,17 @@
       <c r="FQ71" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ71" s="1"/>
+      <c r="GK71" s="1"/>
+      <c r="GL71" s="1"/>
+      <c r="GM71" s="1"/>
+      <c r="GN71" s="1"/>
+      <c r="GO71" s="1"/>
+      <c r="GP71" s="1"/>
+      <c r="GQ71" s="1"/>
+      <c r="GR71" s="1"/>
+      <c r="GS71" s="1"/>
+      <c r="GT71" s="1"/>
       <c r="GU71" s="1" t="s">
         <v>15</v>
       </c>
@@ -58434,6 +59097,17 @@
       <c r="FQ72" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ72" s="1"/>
+      <c r="GK72" s="1"/>
+      <c r="GL72" s="1"/>
+      <c r="GM72" s="1"/>
+      <c r="GN72" s="1"/>
+      <c r="GO72" s="1"/>
+      <c r="GP72" s="1"/>
+      <c r="GQ72" s="1"/>
+      <c r="GR72" s="1"/>
+      <c r="GS72" s="1"/>
+      <c r="GT72" s="1"/>
       <c r="GU72" s="1" t="s">
         <v>15</v>
       </c>
@@ -58640,6 +59314,17 @@
       <c r="FG73" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ73" s="1"/>
+      <c r="GK73" s="1"/>
+      <c r="GL73" s="1"/>
+      <c r="GM73" s="1"/>
+      <c r="GN73" s="1"/>
+      <c r="GO73" s="1"/>
+      <c r="GP73" s="1"/>
+      <c r="GQ73" s="1"/>
+      <c r="GR73" s="1"/>
+      <c r="GS73" s="1"/>
+      <c r="GT73" s="1"/>
       <c r="GU73" s="1" t="s">
         <v>15</v>
       </c>
@@ -58794,6 +59479,17 @@
       <c r="FM74" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ74" s="1"/>
+      <c r="GK74" s="1"/>
+      <c r="GL74" s="1"/>
+      <c r="GM74" s="1"/>
+      <c r="GN74" s="1"/>
+      <c r="GO74" s="1"/>
+      <c r="GP74" s="1"/>
+      <c r="GQ74" s="1"/>
+      <c r="GR74" s="1"/>
+      <c r="GS74" s="1"/>
+      <c r="GT74" s="1"/>
       <c r="GU74" s="1" t="s">
         <v>15</v>
       </c>
@@ -58965,6 +59661,17 @@
       <c r="FM75" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ75" s="1"/>
+      <c r="GK75" s="1"/>
+      <c r="GL75" s="1"/>
+      <c r="GM75" s="1"/>
+      <c r="GN75" s="1"/>
+      <c r="GO75" s="1"/>
+      <c r="GP75" s="1"/>
+      <c r="GQ75" s="1"/>
+      <c r="GR75" s="1"/>
+      <c r="GS75" s="1"/>
+      <c r="GT75" s="1"/>
       <c r="GU75" s="1" t="s">
         <v>15</v>
       </c>
@@ -59101,6 +59808,17 @@
       <c r="FI76" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ76" s="1"/>
+      <c r="GK76" s="1"/>
+      <c r="GL76" s="1"/>
+      <c r="GM76" s="1"/>
+      <c r="GN76" s="1"/>
+      <c r="GO76" s="1"/>
+      <c r="GP76" s="1"/>
+      <c r="GQ76" s="1"/>
+      <c r="GR76" s="1"/>
+      <c r="GS76" s="1"/>
+      <c r="GT76" s="1"/>
       <c r="GU76" s="1" t="s">
         <v>15</v>
       </c>
@@ -59366,6 +60084,17 @@
       <c r="FG77" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ77" s="1"/>
+      <c r="GK77" s="1"/>
+      <c r="GL77" s="1"/>
+      <c r="GM77" s="1"/>
+      <c r="GN77" s="1"/>
+      <c r="GO77" s="1"/>
+      <c r="GP77" s="1"/>
+      <c r="GQ77" s="1"/>
+      <c r="GR77" s="1"/>
+      <c r="GS77" s="1"/>
+      <c r="GT77" s="1"/>
       <c r="GU77" s="1" t="s">
         <v>15</v>
       </c>
@@ -59729,6 +60458,17 @@
       <c r="FG78" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ78" s="1"/>
+      <c r="GK78" s="1"/>
+      <c r="GL78" s="1"/>
+      <c r="GM78" s="1"/>
+      <c r="GN78" s="1"/>
+      <c r="GO78" s="1"/>
+      <c r="GP78" s="1"/>
+      <c r="GQ78" s="1"/>
+      <c r="GR78" s="1"/>
+      <c r="GS78" s="1"/>
+      <c r="GT78" s="1"/>
       <c r="GU78" s="1" t="s">
         <v>15</v>
       </c>
@@ -60075,6 +60815,17 @@
       <c r="FG79" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ79" s="1"/>
+      <c r="GK79" s="1"/>
+      <c r="GL79" s="1"/>
+      <c r="GM79" s="1"/>
+      <c r="GN79" s="1"/>
+      <c r="GO79" s="1"/>
+      <c r="GP79" s="1"/>
+      <c r="GQ79" s="1"/>
+      <c r="GR79" s="1"/>
+      <c r="GS79" s="1"/>
+      <c r="GT79" s="1"/>
       <c r="GU79" s="1" t="s">
         <v>15</v>
       </c>
@@ -60438,6 +61189,17 @@
       <c r="FG80" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ80" s="1"/>
+      <c r="GK80" s="1"/>
+      <c r="GL80" s="1"/>
+      <c r="GM80" s="1"/>
+      <c r="GN80" s="1"/>
+      <c r="GO80" s="1"/>
+      <c r="GP80" s="1"/>
+      <c r="GQ80" s="1"/>
+      <c r="GR80" s="1"/>
+      <c r="GS80" s="1"/>
+      <c r="GT80" s="1"/>
       <c r="GU80" s="1" t="s">
         <v>15</v>
       </c>
@@ -60616,6 +61378,17 @@
       <c r="FG81" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ81" s="1"/>
+      <c r="GK81" s="1"/>
+      <c r="GL81" s="1"/>
+      <c r="GM81" s="1"/>
+      <c r="GN81" s="1"/>
+      <c r="GO81" s="1"/>
+      <c r="GP81" s="1"/>
+      <c r="GQ81" s="1"/>
+      <c r="GR81" s="1"/>
+      <c r="GS81" s="1"/>
+      <c r="GT81" s="1"/>
       <c r="GU81" s="1" t="s">
         <v>15</v>
       </c>
@@ -60715,6 +61488,17 @@
       <c r="FG82" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ82" s="1"/>
+      <c r="GK82" s="1"/>
+      <c r="GL82" s="1"/>
+      <c r="GM82" s="1"/>
+      <c r="GN82" s="1"/>
+      <c r="GO82" s="1"/>
+      <c r="GP82" s="1"/>
+      <c r="GQ82" s="1"/>
+      <c r="GR82" s="1"/>
+      <c r="GS82" s="1"/>
+      <c r="GT82" s="1"/>
       <c r="GU82" s="1" t="s">
         <v>15</v>
       </c>
@@ -61087,6 +61871,17 @@
       <c r="FG84" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ84" s="1"/>
+      <c r="GK84" s="1"/>
+      <c r="GL84" s="1"/>
+      <c r="GM84" s="1"/>
+      <c r="GN84" s="1"/>
+      <c r="GO84" s="1"/>
+      <c r="GP84" s="1"/>
+      <c r="GQ84" s="1"/>
+      <c r="GR84" s="1"/>
+      <c r="GS84" s="1"/>
+      <c r="GT84" s="1"/>
       <c r="GU84" s="1" t="s">
         <v>15</v>
       </c>
@@ -61181,6 +61976,17 @@
       <c r="FG85" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ85" s="1"/>
+      <c r="GK85" s="1"/>
+      <c r="GL85" s="1"/>
+      <c r="GM85" s="1"/>
+      <c r="GN85" s="1"/>
+      <c r="GO85" s="1"/>
+      <c r="GP85" s="1"/>
+      <c r="GQ85" s="1"/>
+      <c r="GR85" s="1"/>
+      <c r="GS85" s="1"/>
+      <c r="GT85" s="1"/>
       <c r="GU85" s="1" t="s">
         <v>15</v>
       </c>
@@ -61290,6 +62096,17 @@
       <c r="FG86" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ86" s="1"/>
+      <c r="GK86" s="1"/>
+      <c r="GL86" s="1"/>
+      <c r="GM86" s="1"/>
+      <c r="GN86" s="1"/>
+      <c r="GO86" s="1"/>
+      <c r="GP86" s="1"/>
+      <c r="GQ86" s="1"/>
+      <c r="GR86" s="1"/>
+      <c r="GS86" s="1"/>
+      <c r="GT86" s="1"/>
       <c r="GU86" s="1" t="s">
         <v>15</v>
       </c>
@@ -61419,6 +62236,17 @@
       <c r="FG87" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ87" s="1"/>
+      <c r="GK87" s="1"/>
+      <c r="GL87" s="1"/>
+      <c r="GM87" s="1"/>
+      <c r="GN87" s="1"/>
+      <c r="GO87" s="1"/>
+      <c r="GP87" s="1"/>
+      <c r="GQ87" s="1"/>
+      <c r="GR87" s="1"/>
+      <c r="GS87" s="1"/>
+      <c r="GT87" s="1"/>
       <c r="GU87" s="1" t="s">
         <v>15</v>
       </c>
@@ -61548,6 +62376,17 @@
       <c r="FG88" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ88" s="1"/>
+      <c r="GK88" s="1"/>
+      <c r="GL88" s="1"/>
+      <c r="GM88" s="1"/>
+      <c r="GN88" s="1"/>
+      <c r="GO88" s="1"/>
+      <c r="GP88" s="1"/>
+      <c r="GQ88" s="1"/>
+      <c r="GR88" s="1"/>
+      <c r="GS88" s="1"/>
+      <c r="GT88" s="1"/>
       <c r="GU88" s="1" t="s">
         <v>15</v>
       </c>
@@ -61677,6 +62516,17 @@
       <c r="FG89" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ89" s="1"/>
+      <c r="GK89" s="1"/>
+      <c r="GL89" s="1"/>
+      <c r="GM89" s="1"/>
+      <c r="GN89" s="1"/>
+      <c r="GO89" s="1"/>
+      <c r="GP89" s="1"/>
+      <c r="GQ89" s="1"/>
+      <c r="GR89" s="1"/>
+      <c r="GS89" s="1"/>
+      <c r="GT89" s="1"/>
       <c r="GU89" s="1" t="s">
         <v>15</v>
       </c>
@@ -61803,6 +62653,17 @@
       <c r="FG90" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ90" s="1"/>
+      <c r="GK90" s="1"/>
+      <c r="GL90" s="1"/>
+      <c r="GM90" s="1"/>
+      <c r="GN90" s="1"/>
+      <c r="GO90" s="1"/>
+      <c r="GP90" s="1"/>
+      <c r="GQ90" s="1"/>
+      <c r="GR90" s="1"/>
+      <c r="GS90" s="1"/>
+      <c r="GT90" s="1"/>
       <c r="GU90" s="1" t="s">
         <v>15</v>
       </c>
@@ -61932,6 +62793,17 @@
       <c r="FG91" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ91" s="1"/>
+      <c r="GK91" s="1"/>
+      <c r="GL91" s="1"/>
+      <c r="GM91" s="1"/>
+      <c r="GN91" s="1"/>
+      <c r="GO91" s="1"/>
+      <c r="GP91" s="1"/>
+      <c r="GQ91" s="1"/>
+      <c r="GR91" s="1"/>
+      <c r="GS91" s="1"/>
+      <c r="GT91" s="1"/>
       <c r="GU91" s="1" t="s">
         <v>15</v>
       </c>
@@ -62061,6 +62933,17 @@
       <c r="FG92" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ92" s="1"/>
+      <c r="GK92" s="1"/>
+      <c r="GL92" s="1"/>
+      <c r="GM92" s="1"/>
+      <c r="GN92" s="1"/>
+      <c r="GO92" s="1"/>
+      <c r="GP92" s="1"/>
+      <c r="GQ92" s="1"/>
+      <c r="GR92" s="1"/>
+      <c r="GS92" s="1"/>
+      <c r="GT92" s="1"/>
       <c r="GU92" s="1" t="s">
         <v>15</v>
       </c>
@@ -62190,6 +63073,17 @@
       <c r="FG93" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ93" s="1"/>
+      <c r="GK93" s="1"/>
+      <c r="GL93" s="1"/>
+      <c r="GM93" s="1"/>
+      <c r="GN93" s="1"/>
+      <c r="GO93" s="1"/>
+      <c r="GP93" s="1"/>
+      <c r="GQ93" s="1"/>
+      <c r="GR93" s="1"/>
+      <c r="GS93" s="1"/>
+      <c r="GT93" s="1"/>
       <c r="GU93" s="1" t="s">
         <v>15</v>
       </c>
@@ -62307,6 +63201,17 @@
       <c r="FG94" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ94" s="1"/>
+      <c r="GK94" s="1"/>
+      <c r="GL94" s="1"/>
+      <c r="GM94" s="1"/>
+      <c r="GN94" s="1"/>
+      <c r="GO94" s="1"/>
+      <c r="GP94" s="1"/>
+      <c r="GQ94" s="1"/>
+      <c r="GR94" s="1"/>
+      <c r="GS94" s="1"/>
+      <c r="GT94" s="1"/>
       <c r="GU94" s="1" t="s">
         <v>15</v>
       </c>
@@ -62424,6 +63329,17 @@
       <c r="FG95" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ95" s="1"/>
+      <c r="GK95" s="1"/>
+      <c r="GL95" s="1"/>
+      <c r="GM95" s="1"/>
+      <c r="GN95" s="1"/>
+      <c r="GO95" s="1"/>
+      <c r="GP95" s="1"/>
+      <c r="GQ95" s="1"/>
+      <c r="GR95" s="1"/>
+      <c r="GS95" s="1"/>
+      <c r="GT95" s="1"/>
       <c r="GU95" s="1" t="s">
         <v>15</v>
       </c>
@@ -62541,6 +63457,17 @@
       <c r="FG96" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ96" s="1"/>
+      <c r="GK96" s="1"/>
+      <c r="GL96" s="1"/>
+      <c r="GM96" s="1"/>
+      <c r="GN96" s="1"/>
+      <c r="GO96" s="1"/>
+      <c r="GP96" s="1"/>
+      <c r="GQ96" s="1"/>
+      <c r="GR96" s="1"/>
+      <c r="GS96" s="1"/>
+      <c r="GT96" s="1"/>
       <c r="GU96" s="1" t="s">
         <v>15</v>
       </c>
@@ -62658,6 +63585,17 @@
       <c r="FG97" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ97" s="1"/>
+      <c r="GK97" s="1"/>
+      <c r="GL97" s="1"/>
+      <c r="GM97" s="1"/>
+      <c r="GN97" s="1"/>
+      <c r="GO97" s="1"/>
+      <c r="GP97" s="1"/>
+      <c r="GQ97" s="1"/>
+      <c r="GR97" s="1"/>
+      <c r="GS97" s="1"/>
+      <c r="GT97" s="1"/>
       <c r="GU97" s="1" t="s">
         <v>15</v>
       </c>
@@ -62775,6 +63713,17 @@
       <c r="FG98" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ98" s="1"/>
+      <c r="GK98" s="1"/>
+      <c r="GL98" s="1"/>
+      <c r="GM98" s="1"/>
+      <c r="GN98" s="1"/>
+      <c r="GO98" s="1"/>
+      <c r="GP98" s="1"/>
+      <c r="GQ98" s="1"/>
+      <c r="GR98" s="1"/>
+      <c r="GS98" s="1"/>
+      <c r="GT98" s="1"/>
       <c r="GU98" s="1" t="s">
         <v>15</v>
       </c>
@@ -62892,6 +63841,17 @@
       <c r="FG99" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ99" s="1"/>
+      <c r="GK99" s="1"/>
+      <c r="GL99" s="1"/>
+      <c r="GM99" s="1"/>
+      <c r="GN99" s="1"/>
+      <c r="GO99" s="1"/>
+      <c r="GP99" s="1"/>
+      <c r="GQ99" s="1"/>
+      <c r="GR99" s="1"/>
+      <c r="GS99" s="1"/>
+      <c r="GT99" s="1"/>
       <c r="GU99" s="1" t="s">
         <v>15</v>
       </c>
@@ -63009,6 +63969,17 @@
       <c r="FG100" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ100" s="1"/>
+      <c r="GK100" s="1"/>
+      <c r="GL100" s="1"/>
+      <c r="GM100" s="1"/>
+      <c r="GN100" s="1"/>
+      <c r="GO100" s="1"/>
+      <c r="GP100" s="1"/>
+      <c r="GQ100" s="1"/>
+      <c r="GR100" s="1"/>
+      <c r="GS100" s="1"/>
+      <c r="GT100" s="1"/>
       <c r="GU100" s="1" t="s">
         <v>15</v>
       </c>
@@ -63126,6 +64097,17 @@
       <c r="FG101" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ101" s="1"/>
+      <c r="GK101" s="1"/>
+      <c r="GL101" s="1"/>
+      <c r="GM101" s="1"/>
+      <c r="GN101" s="1"/>
+      <c r="GO101" s="1"/>
+      <c r="GP101" s="1"/>
+      <c r="GQ101" s="1"/>
+      <c r="GR101" s="1"/>
+      <c r="GS101" s="1"/>
+      <c r="GT101" s="1"/>
       <c r="GU101" s="1" t="s">
         <v>15</v>
       </c>
@@ -63240,6 +64222,17 @@
       <c r="FG102" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ102" s="1"/>
+      <c r="GK102" s="1"/>
+      <c r="GL102" s="1"/>
+      <c r="GM102" s="1"/>
+      <c r="GN102" s="1"/>
+      <c r="GO102" s="1"/>
+      <c r="GP102" s="1"/>
+      <c r="GQ102" s="1"/>
+      <c r="GR102" s="1"/>
+      <c r="GS102" s="1"/>
+      <c r="GT102" s="1"/>
       <c r="GU102" s="1" t="s">
         <v>15</v>
       </c>
@@ -63337,6 +64330,17 @@
       <c r="FG103" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ103" s="1"/>
+      <c r="GK103" s="1"/>
+      <c r="GL103" s="1"/>
+      <c r="GM103" s="1"/>
+      <c r="GN103" s="1"/>
+      <c r="GO103" s="1"/>
+      <c r="GP103" s="1"/>
+      <c r="GQ103" s="1"/>
+      <c r="GR103" s="1"/>
+      <c r="GS103" s="1"/>
+      <c r="GT103" s="1"/>
       <c r="GU103" s="1" t="s">
         <v>15</v>
       </c>
@@ -63434,6 +64438,17 @@
       <c r="FG104" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ104" s="1"/>
+      <c r="GK104" s="1"/>
+      <c r="GL104" s="1"/>
+      <c r="GM104" s="1"/>
+      <c r="GN104" s="1"/>
+      <c r="GO104" s="1"/>
+      <c r="GP104" s="1"/>
+      <c r="GQ104" s="1"/>
+      <c r="GR104" s="1"/>
+      <c r="GS104" s="1"/>
+      <c r="GT104" s="1"/>
       <c r="GU104" s="1" t="s">
         <v>15</v>
       </c>
@@ -63531,6 +64546,17 @@
       <c r="FG105" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ105" s="1"/>
+      <c r="GK105" s="1"/>
+      <c r="GL105" s="1"/>
+      <c r="GM105" s="1"/>
+      <c r="GN105" s="1"/>
+      <c r="GO105" s="1"/>
+      <c r="GP105" s="1"/>
+      <c r="GQ105" s="1"/>
+      <c r="GR105" s="1"/>
+      <c r="GS105" s="1"/>
+      <c r="GT105" s="1"/>
       <c r="GU105" s="1" t="s">
         <v>15</v>
       </c>
@@ -63628,6 +64654,17 @@
       <c r="FG106" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ106" s="1"/>
+      <c r="GK106" s="1"/>
+      <c r="GL106" s="1"/>
+      <c r="GM106" s="1"/>
+      <c r="GN106" s="1"/>
+      <c r="GO106" s="1"/>
+      <c r="GP106" s="1"/>
+      <c r="GQ106" s="1"/>
+      <c r="GR106" s="1"/>
+      <c r="GS106" s="1"/>
+      <c r="GT106" s="1"/>
       <c r="GU106" s="1" t="s">
         <v>15</v>
       </c>
@@ -63725,6 +64762,17 @@
       <c r="FG107" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ107" s="1"/>
+      <c r="GK107" s="1"/>
+      <c r="GL107" s="1"/>
+      <c r="GM107" s="1"/>
+      <c r="GN107" s="1"/>
+      <c r="GO107" s="1"/>
+      <c r="GP107" s="1"/>
+      <c r="GQ107" s="1"/>
+      <c r="GR107" s="1"/>
+      <c r="GS107" s="1"/>
+      <c r="GT107" s="1"/>
       <c r="GU107" s="1" t="s">
         <v>15</v>
       </c>
@@ -63822,6 +64870,17 @@
       <c r="FG108" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ108" s="1"/>
+      <c r="GK108" s="1"/>
+      <c r="GL108" s="1"/>
+      <c r="GM108" s="1"/>
+      <c r="GN108" s="1"/>
+      <c r="GO108" s="1"/>
+      <c r="GP108" s="1"/>
+      <c r="GQ108" s="1"/>
+      <c r="GR108" s="1"/>
+      <c r="GS108" s="1"/>
+      <c r="GT108" s="1"/>
       <c r="GU108" s="1" t="s">
         <v>15</v>
       </c>
@@ -63919,6 +64978,17 @@
       <c r="FG109" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ109" s="1"/>
+      <c r="GK109" s="1"/>
+      <c r="GL109" s="1"/>
+      <c r="GM109" s="1"/>
+      <c r="GN109" s="1"/>
+      <c r="GO109" s="1"/>
+      <c r="GP109" s="1"/>
+      <c r="GQ109" s="1"/>
+      <c r="GR109" s="1"/>
+      <c r="GS109" s="1"/>
+      <c r="GT109" s="1"/>
       <c r="GU109" s="1" t="s">
         <v>15</v>
       </c>
@@ -64016,6 +65086,17 @@
       <c r="FG110" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ110" s="1"/>
+      <c r="GK110" s="1"/>
+      <c r="GL110" s="1"/>
+      <c r="GM110" s="1"/>
+      <c r="GN110" s="1"/>
+      <c r="GO110" s="1"/>
+      <c r="GP110" s="1"/>
+      <c r="GQ110" s="1"/>
+      <c r="GR110" s="1"/>
+      <c r="GS110" s="1"/>
+      <c r="GT110" s="1"/>
       <c r="GU110" s="1" t="s">
         <v>15</v>
       </c>
@@ -64113,6 +65194,17 @@
       <c r="FG111" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ111" s="1"/>
+      <c r="GK111" s="1"/>
+      <c r="GL111" s="1"/>
+      <c r="GM111" s="1"/>
+      <c r="GN111" s="1"/>
+      <c r="GO111" s="1"/>
+      <c r="GP111" s="1"/>
+      <c r="GQ111" s="1"/>
+      <c r="GR111" s="1"/>
+      <c r="GS111" s="1"/>
+      <c r="GT111" s="1"/>
       <c r="GU111" s="1" t="s">
         <v>15</v>
       </c>
@@ -64210,6 +65302,17 @@
       <c r="FG112" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ112" s="1"/>
+      <c r="GK112" s="1"/>
+      <c r="GL112" s="1"/>
+      <c r="GM112" s="1"/>
+      <c r="GN112" s="1"/>
+      <c r="GO112" s="1"/>
+      <c r="GP112" s="1"/>
+      <c r="GQ112" s="1"/>
+      <c r="GR112" s="1"/>
+      <c r="GS112" s="1"/>
+      <c r="GT112" s="1"/>
       <c r="GU112" s="1" t="s">
         <v>15</v>
       </c>
@@ -64307,6 +65410,17 @@
       <c r="FG113" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ113" s="1"/>
+      <c r="GK113" s="1"/>
+      <c r="GL113" s="1"/>
+      <c r="GM113" s="1"/>
+      <c r="GN113" s="1"/>
+      <c r="GO113" s="1"/>
+      <c r="GP113" s="1"/>
+      <c r="GQ113" s="1"/>
+      <c r="GR113" s="1"/>
+      <c r="GS113" s="1"/>
+      <c r="GT113" s="1"/>
       <c r="GU113" s="1" t="s">
         <v>15</v>
       </c>
@@ -64404,6 +65518,17 @@
       <c r="FG114" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ114" s="1"/>
+      <c r="GK114" s="1"/>
+      <c r="GL114" s="1"/>
+      <c r="GM114" s="1"/>
+      <c r="GN114" s="1"/>
+      <c r="GO114" s="1"/>
+      <c r="GP114" s="1"/>
+      <c r="GQ114" s="1"/>
+      <c r="GR114" s="1"/>
+      <c r="GS114" s="1"/>
+      <c r="GT114" s="1"/>
       <c r="GU114" s="1" t="s">
         <v>15</v>
       </c>
@@ -64501,6 +65626,17 @@
       <c r="FG115" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ115" s="1"/>
+      <c r="GK115" s="1"/>
+      <c r="GL115" s="1"/>
+      <c r="GM115" s="1"/>
+      <c r="GN115" s="1"/>
+      <c r="GO115" s="1"/>
+      <c r="GP115" s="1"/>
+      <c r="GQ115" s="1"/>
+      <c r="GR115" s="1"/>
+      <c r="GS115" s="1"/>
+      <c r="GT115" s="1"/>
       <c r="GU115" s="1" t="s">
         <v>15</v>
       </c>
@@ -64613,6 +65749,17 @@
       <c r="FG116" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ116" s="1"/>
+      <c r="GK116" s="1"/>
+      <c r="GL116" s="1"/>
+      <c r="GM116" s="1"/>
+      <c r="GN116" s="1"/>
+      <c r="GO116" s="1"/>
+      <c r="GP116" s="1"/>
+      <c r="GQ116" s="1"/>
+      <c r="GR116" s="1"/>
+      <c r="GS116" s="1"/>
+      <c r="GT116" s="1"/>
       <c r="GU116" s="1" t="s">
         <v>15</v>
       </c>
@@ -64742,6 +65889,17 @@
       <c r="FG117" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ117" s="1"/>
+      <c r="GK117" s="1"/>
+      <c r="GL117" s="1"/>
+      <c r="GM117" s="1"/>
+      <c r="GN117" s="1"/>
+      <c r="GO117" s="1"/>
+      <c r="GP117" s="1"/>
+      <c r="GQ117" s="1"/>
+      <c r="GR117" s="1"/>
+      <c r="GS117" s="1"/>
+      <c r="GT117" s="1"/>
       <c r="GU117" s="1" t="s">
         <v>15</v>
       </c>
@@ -64871,6 +66029,17 @@
       <c r="FG118" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="GJ118" s="1"/>
+      <c r="GK118" s="1"/>
+      <c r="GL118" s="1"/>
+      <c r="GM118" s="1"/>
+      <c r="GN118" s="1"/>
+      <c r="GO118" s="1"/>
+      <c r="GP118" s="1"/>
+      <c r="GQ118" s="1"/>
+      <c r="GR118" s="1"/>
+      <c r="GS118" s="1"/>
+      <c r="GT118" s="1"/>
       <c r="GU118" s="1" t="s">
         <v>15</v>
       </c>
@@ -64970,6 +66139,17 @@
       <c r="JO118" s="1"/>
     </row>
     <row r="119">
+      <c r="GJ119" s="1"/>
+      <c r="GK119" s="1"/>
+      <c r="GL119" s="1"/>
+      <c r="GM119" s="1"/>
+      <c r="GN119" s="1"/>
+      <c r="GO119" s="1"/>
+      <c r="GP119" s="1"/>
+      <c r="GQ119" s="1"/>
+      <c r="GR119" s="1"/>
+      <c r="GS119" s="1"/>
+      <c r="GT119" s="1"/>
       <c r="HK119" s="1"/>
       <c r="HL119" s="1"/>
       <c r="HM119" s="1"/>

</xml_diff>

<commit_message>
Revised linen item list at various locations
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -38741,6 +38741,9 @@
       <c r="C8" s="2" t="s">
         <v>941</v>
       </c>
+      <c r="N8" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FG8" s="1" t="s">
         <v>15</v>
       </c>
@@ -38846,6 +38849,9 @@
       <c r="C9" s="2" t="s">
         <v>941</v>
       </c>
+      <c r="N9" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FG9" s="1" t="s">
         <v>15</v>
       </c>
@@ -39275,6 +39281,9 @@
       <c r="C13" s="2" t="s">
         <v>941</v>
       </c>
+      <c r="N13" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FG13" s="1" t="s">
         <v>15</v>
       </c>
@@ -39380,6 +39389,9 @@
       <c r="C14" s="2" t="s">
         <v>941</v>
       </c>
+      <c r="N14" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FG14" s="1" t="s">
         <v>15</v>
       </c>
@@ -39488,9 +39500,6 @@
       <c r="G15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="N15" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="FG15" s="1" t="s">
         <v>15</v>
       </c>
@@ -39599,9 +39608,6 @@
       <c r="G16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="N16" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="FG16" s="1" t="s">
         <v>15</v>
       </c>
@@ -39710,9 +39716,6 @@
       <c r="G17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="N17" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="FG17" s="1" t="s">
         <v>15</v>
       </c>
@@ -39845,6 +39848,9 @@
       <c r="CM18" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CN18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CO18" s="1" t="s">
         <v>15</v>
       </c>
@@ -39857,6 +39863,9 @@
       <c r="CU18" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CV18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CW18" s="1" t="s">
         <v>15</v>
       </c>
@@ -39869,6 +39878,9 @@
       <c r="DC18" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DD18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DE18" s="1" t="s">
         <v>15</v>
       </c>
@@ -39881,6 +39893,9 @@
       <c r="DK18" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DL18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DM18" s="1" t="s">
         <v>15</v>
       </c>
@@ -39893,6 +39908,9 @@
       <c r="DS18" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DT18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DU18" s="1" t="s">
         <v>15</v>
       </c>
@@ -39903,6 +39921,9 @@
         <v>15</v>
       </c>
       <c r="EA18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="EB18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EC18" s="1" t="s">
@@ -40077,7 +40098,9 @@
       <c r="HJ18" s="1"/>
       <c r="HK18" s="1"/>
       <c r="HL18" s="1"/>
-      <c r="HM18" s="1"/>
+      <c r="HM18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HN18" s="1" t="s">
         <v>15</v>
       </c>
@@ -40096,7 +40119,9 @@
       <c r="HU18" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="HV18" s="1"/>
+      <c r="HV18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HW18" s="1" t="s">
         <v>15</v>
       </c>
@@ -40108,7 +40133,9 @@
       <c r="IA18" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IB18" s="1"/>
+      <c r="IB18" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IC18" s="1" t="s">
         <v>15</v>
       </c>
@@ -40389,6 +40416,9 @@
       <c r="CQ19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CR19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CS19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40401,6 +40431,9 @@
       <c r="CY19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CZ19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DA19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40413,6 +40446,9 @@
       <c r="DG19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DH19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DI19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40425,6 +40461,9 @@
       <c r="DO19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DP19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DQ19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40437,6 +40476,9 @@
       <c r="DW19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DX19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DY19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40449,40 +40491,61 @@
       <c r="EE19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EF19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EG19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EJ19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EK19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EL19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EN19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EO19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EP19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="ER19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="ES19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="ET19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EV19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EW19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EX19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EZ19" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="FA19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FB19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="FD19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="FE19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="FF19" s="1" t="s">
@@ -40663,7 +40726,9 @@
       <c r="HP19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="HQ19" s="1"/>
+      <c r="HQ19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HR19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40678,7 +40743,9 @@
       <c r="HY19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="HZ19" s="1"/>
+      <c r="HZ19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IA19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40690,7 +40757,9 @@
       <c r="IE19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IF19" s="1"/>
+      <c r="IF19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IG19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40698,7 +40767,9 @@
       <c r="II19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IJ19" s="1"/>
+      <c r="IJ19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IK19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40706,7 +40777,9 @@
       <c r="IM19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IN19" s="1"/>
+      <c r="IN19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IO19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40714,7 +40787,9 @@
       <c r="IQ19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IR19" s="1"/>
+      <c r="IR19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IS19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40722,7 +40797,9 @@
       <c r="IU19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IV19" s="1"/>
+      <c r="IV19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IW19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40730,7 +40807,9 @@
       <c r="IY19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IZ19" s="1"/>
+      <c r="IZ19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JA19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40738,7 +40817,9 @@
       <c r="JC19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="JD19" s="1"/>
+      <c r="JD19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JE19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40746,7 +40827,9 @@
       <c r="JG19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="JH19" s="1"/>
+      <c r="JH19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JI19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40754,7 +40837,9 @@
       <c r="JK19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="JL19" s="1"/>
+      <c r="JL19" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JM19" s="1" t="s">
         <v>15</v>
       </c>
@@ -40804,39 +40889,16 @@
       <c r="FQ20" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="GJ20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GK20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GL20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GM20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GN20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GO20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GP20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GQ20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GR20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GS20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="GT20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="GK20" s="1"/>
+      <c r="GL20" s="1"/>
+      <c r="GM20" s="1"/>
+      <c r="GN20" s="1"/>
+      <c r="GO20" s="1"/>
+      <c r="GP20" s="1"/>
+      <c r="GQ20" s="1"/>
+      <c r="GR20" s="1"/>
+      <c r="GS20" s="1"/>
+      <c r="GT20" s="1"/>
       <c r="GU20" s="1" t="s">
         <v>15</v>
       </c>
@@ -40882,9 +40944,7 @@
       <c r="HM20" s="1"/>
       <c r="HN20" s="1"/>
       <c r="HO20" s="1"/>
-      <c r="HP20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="HP20" s="1"/>
       <c r="HQ20" s="1"/>
       <c r="HR20" s="1"/>
       <c r="HS20" s="1" t="s">
@@ -40897,65 +40957,45 @@
       <c r="HV20" s="1"/>
       <c r="HW20" s="1"/>
       <c r="HX20" s="1"/>
-      <c r="HY20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="HY20" s="1"/>
       <c r="HZ20" s="1"/>
       <c r="IA20" s="1"/>
       <c r="IB20" s="1"/>
       <c r="IC20" s="1"/>
       <c r="ID20" s="1"/>
-      <c r="IE20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IE20" s="1"/>
       <c r="IF20" s="1"/>
       <c r="IG20" s="1"/>
       <c r="IH20" s="1"/>
-      <c r="II20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="II20" s="1"/>
       <c r="IJ20" s="1"/>
       <c r="IK20" s="1"/>
       <c r="IL20" s="1"/>
-      <c r="IM20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IM20" s="1"/>
       <c r="IN20" s="1"/>
       <c r="IO20" s="1"/>
       <c r="IP20" s="1"/>
-      <c r="IQ20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IQ20" s="1"/>
       <c r="IR20" s="1"/>
       <c r="IS20" s="1"/>
       <c r="IT20" s="1"/>
-      <c r="IU20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IU20" s="1"/>
       <c r="IV20" s="1"/>
       <c r="IW20" s="1"/>
       <c r="IX20" s="1"/>
-      <c r="IY20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="IY20" s="1"/>
       <c r="IZ20" s="1"/>
       <c r="JA20" s="1"/>
       <c r="JB20" s="1"/>
-      <c r="JC20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="JC20" s="1"/>
       <c r="JD20" s="1"/>
       <c r="JE20" s="1"/>
       <c r="JF20" s="1"/>
-      <c r="JG20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="JG20" s="1"/>
       <c r="JH20" s="1"/>
       <c r="JI20" s="1"/>
       <c r="JJ20" s="1"/>
-      <c r="JK20" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="JK20" s="1"/>
       <c r="JL20" s="1"/>
       <c r="JM20" s="1"/>
       <c r="JN20" s="1"/>
@@ -41600,60 +41640,168 @@
       <c r="CM22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CN22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CO22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CQ22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CR22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CS22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CU22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CV22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CW22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CY22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CZ22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="DA22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DC22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DD22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="DE22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DG22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DH22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="DI22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DK22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DL22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="DM22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DO22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DP22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="DQ22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DS22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DT22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="DU22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DW22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DX22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="DY22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EA22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EB22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="EC22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EE22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EF22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="EG22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EH22" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EJ22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EK22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="EL22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EN22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EO22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="EP22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="ER22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="ES22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="ET22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EV22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EW22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="EX22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EZ22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="FA22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="FB22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FD22" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="FE22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="FF22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FG22" s="1" t="s">
         <v>15</v>
       </c>
@@ -41819,14 +41967,22 @@
       <c r="HL22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="HM22" s="1"/>
-      <c r="HN22" s="1"/>
+      <c r="HM22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="HN22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HO22" s="1"/>
       <c r="HP22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="HQ22" s="1"/>
-      <c r="HR22" s="1"/>
+      <c r="HQ22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="HR22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HS22" s="1" t="s">
         <v>15</v>
       </c>
@@ -41834,70 +41990,118 @@
       <c r="HU22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="HV22" s="1"/>
-      <c r="HW22" s="1"/>
+      <c r="HV22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="HW22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HX22" s="1"/>
       <c r="HY22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="HZ22" s="1"/>
-      <c r="IA22" s="1"/>
-      <c r="IB22" s="1"/>
-      <c r="IC22" s="1"/>
+      <c r="HZ22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IA22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IB22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IC22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="ID22" s="1"/>
       <c r="IE22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IF22" s="1"/>
-      <c r="IG22" s="1"/>
+      <c r="IF22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IG22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IH22" s="1"/>
       <c r="II22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IJ22" s="1"/>
-      <c r="IK22" s="1"/>
+      <c r="IJ22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IK22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IL22" s="1"/>
       <c r="IM22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IN22" s="1"/>
-      <c r="IO22" s="1"/>
+      <c r="IN22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IO22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IP22" s="1"/>
       <c r="IQ22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IR22" s="1"/>
-      <c r="IS22" s="1"/>
+      <c r="IR22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IS22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IT22" s="1"/>
       <c r="IU22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IV22" s="1"/>
-      <c r="IW22" s="1"/>
+      <c r="IV22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IW22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IX22" s="1"/>
       <c r="IY22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IZ22" s="1"/>
-      <c r="JA22" s="1"/>
+      <c r="IZ22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="JA22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JB22" s="1"/>
       <c r="JC22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="JD22" s="1"/>
-      <c r="JE22" s="1"/>
+      <c r="JD22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="JE22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JF22" s="1"/>
       <c r="JG22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="JH22" s="1"/>
-      <c r="JI22" s="1"/>
+      <c r="JH22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="JI22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JJ22" s="1"/>
       <c r="JK22" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="JL22" s="1"/>
-      <c r="JM22" s="1"/>
+      <c r="JL22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="JM22" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JN22" s="1"/>
       <c r="JO22" s="1"/>
     </row>
@@ -41992,108 +42196,162 @@
       <c r="CM23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CN23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CO23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="CQ23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CR23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CS23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="CU23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CV23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CW23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="CY23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CZ23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DA23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="DC23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DD23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DE23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="DG23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DH23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DI23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="DK23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DL23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DM23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="DO23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DP23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DQ23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="DS23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DT23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DU23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="DW23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="DX23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="DY23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EA23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EB23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EC23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EE23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EF23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EG23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EJ23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EK23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EL23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EN23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EO23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EP23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="ER23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="ES23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="ET23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EV23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="EW23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="EX23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="EZ23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="FA23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FB23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="FD23" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="FE23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FF23" s="1" t="s">
         <v>15</v>
       </c>
@@ -42181,17 +42439,39 @@
       <c r="GI23" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="GJ23" s="1"/>
-      <c r="GK23" s="1"/>
-      <c r="GL23" s="1"/>
-      <c r="GM23" s="1"/>
-      <c r="GN23" s="1"/>
-      <c r="GO23" s="1"/>
-      <c r="GP23" s="1"/>
-      <c r="GQ23" s="1"/>
-      <c r="GR23" s="1"/>
-      <c r="GS23" s="1"/>
-      <c r="GT23" s="1"/>
+      <c r="GJ23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GK23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GL23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GM23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GN23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GO23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GP23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GQ23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GR23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GS23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="GT23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="GU23" s="1" t="s">
         <v>15</v>
       </c>
@@ -42237,13 +42517,19 @@
       <c r="HJ23" s="1"/>
       <c r="HK23" s="1"/>
       <c r="HL23" s="1"/>
-      <c r="HM23" s="1"/>
+      <c r="HM23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HN23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="HO23" s="1"/>
-      <c r="HP23" s="1"/>
-      <c r="HQ23" s="1"/>
+      <c r="HP23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="HQ23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HR23" s="1" t="s">
         <v>15</v>
       </c>
@@ -42254,71 +42540,115 @@
       <c r="HU23" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="HV23" s="1"/>
+      <c r="HV23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="HW23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="HX23" s="1"/>
-      <c r="HY23" s="1"/>
-      <c r="HZ23" s="1"/>
+      <c r="HY23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="HZ23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IA23" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="IB23" s="1"/>
+      <c r="IB23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IC23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="ID23" s="1"/>
-      <c r="IE23" s="1"/>
-      <c r="IF23" s="1"/>
+      <c r="IE23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IF23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IG23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IH23" s="1"/>
-      <c r="II23" s="1"/>
-      <c r="IJ23" s="1"/>
+      <c r="II23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IJ23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IK23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IL23" s="1"/>
-      <c r="IM23" s="1"/>
-      <c r="IN23" s="1"/>
+      <c r="IM23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IN23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IO23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IP23" s="1"/>
-      <c r="IQ23" s="1"/>
-      <c r="IR23" s="1"/>
+      <c r="IQ23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IR23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IS23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IT23" s="1"/>
-      <c r="IU23" s="1"/>
-      <c r="IV23" s="1"/>
+      <c r="IU23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IV23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="IW23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="IX23" s="1"/>
-      <c r="IY23" s="1"/>
-      <c r="IZ23" s="1"/>
+      <c r="IY23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="IZ23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JA23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JB23" s="1"/>
-      <c r="JC23" s="1"/>
-      <c r="JD23" s="1"/>
+      <c r="JC23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="JD23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JE23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JF23" s="1"/>
-      <c r="JG23" s="1"/>
-      <c r="JH23" s="1"/>
+      <c r="JG23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="JH23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JI23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="JJ23" s="1"/>
-      <c r="JK23" s="1"/>
-      <c r="JL23" s="1"/>
+      <c r="JK23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="JL23" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="JM23" s="1" t="s">
         <v>15</v>
       </c>
@@ -42366,6 +42696,9 @@
         <v>15</v>
       </c>
       <c r="Y24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD24" s="1" t="s">
         <v>15</v>
       </c>
       <c r="AI24" s="1" t="s">
@@ -42530,9 +42863,6 @@
       <c r="C25" s="2" t="s">
         <v>958</v>
       </c>
-      <c r="AD25" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="BP25" s="1" t="s">
         <v>15</v>
       </c>
@@ -46302,6 +46632,12 @@
       <c r="C46" s="2" t="s">
         <v>985</v>
       </c>
+      <c r="D46" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Z46" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="AT46" s="1" t="s">
         <v>15</v>
       </c>
@@ -49227,6 +49563,12 @@
       <c r="C52" s="2" t="s">
         <v>985</v>
       </c>
+      <c r="D52" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Z52" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="AT52" s="1" t="s">
         <v>15</v>
       </c>
@@ -52176,6 +52518,12 @@
       <c r="I58" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="K58" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Z58" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="AT58" s="1" t="s">
         <v>15</v>
       </c>
@@ -53162,12 +53510,6 @@
       <c r="C60" s="2" t="s">
         <v>985</v>
       </c>
-      <c r="H60" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I60" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="Q60" s="1" t="s">
         <v>15</v>
       </c>
@@ -54154,12 +54496,6 @@
       <c r="C62" s="2" t="s">
         <v>985</v>
       </c>
-      <c r="H62" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I62" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="Q62" s="1" t="s">
         <v>15</v>
       </c>
@@ -54665,12 +55001,6 @@
       <c r="C63" s="2" t="s">
         <v>985</v>
       </c>
-      <c r="H63" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I63" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="AV63" s="1" t="s">
         <v>15</v>
       </c>
@@ -55125,6 +55455,12 @@
       <c r="I64" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="K64" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Z64" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="AT64" s="1" t="s">
         <v>15</v>
       </c>
@@ -57060,6 +57396,12 @@
       </c>
       <c r="C68" s="2" t="s">
         <v>1010</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="Z68" s="1" t="s">
         <v>15</v>
@@ -63704,6 +64046,12 @@
       <c r="C98" s="2" t="s">
         <v>1031</v>
       </c>
+      <c r="H98" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="AP98" s="1" t="s">
         <v>15</v>
       </c>
@@ -63832,6 +64180,12 @@
       <c r="C99" s="2" t="s">
         <v>1031</v>
       </c>
+      <c r="H99" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="AP99" s="1" t="s">
         <v>15</v>
       </c>
@@ -63960,6 +64314,12 @@
       <c r="C100" s="2" t="s">
         <v>1031</v>
       </c>
+      <c r="H100" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="AP100" s="1" t="s">
         <v>15</v>
       </c>
@@ -64087,6 +64447,12 @@
       </c>
       <c r="C101" s="2" t="s">
         <v>1031</v>
+      </c>
+      <c r="H101" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="AP101" s="1" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Additional items for linen inventory locations
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -43526,6 +43526,9 @@
       <c r="C31" s="2" t="s">
         <v>967</v>
       </c>
+      <c r="AR31" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="FG31" s="1" t="s">
         <v>15</v>
       </c>
@@ -56925,6 +56928,9 @@
       <c r="BI67" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="BK67" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="BO67" s="1" t="s">
         <v>15</v>
       </c>
@@ -56961,7 +56967,22 @@
       <c r="CD67" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CE67" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CF67" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CG67" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CH67" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CI67" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CJ67" s="1" t="s">
         <v>15</v>
       </c>
       <c r="CL67" s="1" t="s">
@@ -57439,6 +57460,9 @@
       <c r="BH68" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="BK68" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="BO68" s="1" t="s">
         <v>15</v>
       </c>
@@ -57451,7 +57475,22 @@
       <c r="CD68" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CE68" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CF68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CG68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CH68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CI68" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CJ68" s="1" t="s">
         <v>15</v>
       </c>
       <c r="CL68" s="1" t="s">
@@ -57890,6 +57929,9 @@
       <c r="BI69" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="BK69" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="BO69" s="1" t="s">
         <v>15</v>
       </c>
@@ -57920,7 +57962,22 @@
       <c r="CD69" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CE69" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CF69" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CG69" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CH69" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CI69" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CJ69" s="1" t="s">
         <v>15</v>
       </c>
       <c r="CK69" s="1" t="s">
@@ -58357,6 +58414,9 @@
       <c r="BI70" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="BK70" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="BO70" s="1" t="s">
         <v>15</v>
       </c>
@@ -58387,7 +58447,22 @@
       <c r="CD70" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="CE70" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="CF70" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CG70" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CH70" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CI70" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CJ70" s="1" t="s">
         <v>15</v>
       </c>
       <c r="CK70" s="1" t="s">
@@ -58827,6 +58902,9 @@
       <c r="BI71" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="BK71" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="BO71" s="1" t="s">
         <v>15</v>
       </c>
@@ -59239,6 +59317,9 @@
         <v>15</v>
       </c>
       <c r="BE72" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="BK72" s="1" t="s">
         <v>15</v>
       </c>
       <c r="BO72" s="1" t="s">

</xml_diff>

<commit_message>
Add persistent login, performance improvements and issue history
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="8"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -6806,7 +6806,7 @@
         <v>85</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>14</v>
@@ -20075,7 +20075,7 @@
         <v>178</v>
       </c>
       <c r="D2" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>179</v>
@@ -20101,7 +20101,7 @@
         <v>182</v>
       </c>
       <c r="D3" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>179</v>
@@ -20127,7 +20127,7 @@
         <v>184</v>
       </c>
       <c r="D4" s="1">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>179</v>
@@ -20153,7 +20153,7 @@
         <v>178</v>
       </c>
       <c r="D5" s="1">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>179</v>
@@ -20179,7 +20179,7 @@
         <v>182</v>
       </c>
       <c r="D6" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>179</v>
@@ -20205,7 +20205,7 @@
         <v>190</v>
       </c>
       <c r="D7" s="1">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>179</v>
@@ -20231,7 +20231,7 @@
         <v>184</v>
       </c>
       <c r="D8" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>179</v>
@@ -20257,7 +20257,7 @@
         <v>192</v>
       </c>
       <c r="D9" s="1">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>179</v>
@@ -20283,7 +20283,7 @@
         <v>192</v>
       </c>
       <c r="D10" s="1">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>179</v>
@@ -20309,7 +20309,7 @@
         <v>178</v>
       </c>
       <c r="D11" s="1">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>179</v>
@@ -20335,7 +20335,7 @@
         <v>182</v>
       </c>
       <c r="D12" s="1">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>179</v>
@@ -20361,7 +20361,7 @@
         <v>190</v>
       </c>
       <c r="D13" s="1">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>179</v>
@@ -20387,7 +20387,7 @@
         <v>182</v>
       </c>
       <c r="D14" s="1">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>179</v>
@@ -20413,7 +20413,7 @@
         <v>182</v>
       </c>
       <c r="D15" s="1">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>179</v>
@@ -20439,7 +20439,7 @@
         <v>190</v>
       </c>
       <c r="D16" s="1">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>179</v>
@@ -20465,7 +20465,7 @@
         <v>182</v>
       </c>
       <c r="D17" s="1">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>179</v>
@@ -20491,7 +20491,7 @@
         <v>192</v>
       </c>
       <c r="D18" s="1">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>179</v>
@@ -20517,7 +20517,7 @@
         <v>178</v>
       </c>
       <c r="D19" s="1">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>179</v>
@@ -20543,7 +20543,7 @@
         <v>178</v>
       </c>
       <c r="D20" s="1">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>179</v>
@@ -20569,7 +20569,7 @@
         <v>178</v>
       </c>
       <c r="D21" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>179</v>
@@ -20595,7 +20595,7 @@
         <v>178</v>
       </c>
       <c r="D22" s="1">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>179</v>
@@ -20621,7 +20621,7 @@
         <v>178</v>
       </c>
       <c r="D23" s="1">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>179</v>
@@ -20647,7 +20647,7 @@
         <v>182</v>
       </c>
       <c r="D24" s="1">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>179</v>
@@ -20673,7 +20673,7 @@
         <v>178</v>
       </c>
       <c r="D25" s="1">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>179</v>
@@ -20699,7 +20699,7 @@
         <v>178</v>
       </c>
       <c r="D26" s="1">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>179</v>
@@ -20725,7 +20725,7 @@
         <v>178</v>
       </c>
       <c r="D27" s="1">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>179</v>
@@ -20751,7 +20751,7 @@
         <v>182</v>
       </c>
       <c r="D28" s="1">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>179</v>
@@ -20777,7 +20777,7 @@
         <v>192</v>
       </c>
       <c r="D29" s="1">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>179</v>
@@ -20803,7 +20803,7 @@
         <v>184</v>
       </c>
       <c r="D30" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>225</v>
@@ -20829,7 +20829,7 @@
         <v>89</v>
       </c>
       <c r="D31" s="1">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>225</v>
@@ -20855,7 +20855,7 @@
         <v>184</v>
       </c>
       <c r="D32" s="1">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>225</v>
@@ -20881,7 +20881,7 @@
         <v>184</v>
       </c>
       <c r="D33" s="1">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>225</v>
@@ -20907,7 +20907,7 @@
         <v>178</v>
       </c>
       <c r="D34" s="1">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>225</v>
@@ -20933,7 +20933,7 @@
         <v>184</v>
       </c>
       <c r="D35" s="1">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>225</v>
@@ -20959,7 +20959,7 @@
         <v>184</v>
       </c>
       <c r="D36" s="1">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>225</v>
@@ -20985,7 +20985,7 @@
         <v>184</v>
       </c>
       <c r="D37" s="1">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>225</v>
@@ -21011,7 +21011,7 @@
         <v>184</v>
       </c>
       <c r="D38" s="1">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>225</v>
@@ -21037,7 +21037,7 @@
         <v>184</v>
       </c>
       <c r="D39" s="1">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>225</v>
@@ -21089,7 +21089,7 @@
         <v>184</v>
       </c>
       <c r="D41" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>225</v>
@@ -21115,7 +21115,7 @@
         <v>184</v>
       </c>
       <c r="D42" s="1">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>225</v>
@@ -21141,7 +21141,7 @@
         <v>184</v>
       </c>
       <c r="D43" s="1">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>225</v>
@@ -21167,7 +21167,7 @@
         <v>184</v>
       </c>
       <c r="D44" s="1">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>225</v>
@@ -21219,7 +21219,7 @@
         <v>184</v>
       </c>
       <c r="D46" s="1">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>225</v>
@@ -21245,7 +21245,7 @@
         <v>184</v>
       </c>
       <c r="D47" s="1">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>225</v>
@@ -21271,7 +21271,7 @@
         <v>184</v>
       </c>
       <c r="D48" s="1">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>225</v>
@@ -21297,7 +21297,7 @@
         <v>184</v>
       </c>
       <c r="D49" s="1">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>225</v>
@@ -21323,7 +21323,7 @@
         <v>182</v>
       </c>
       <c r="D50" s="1">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>239</v>
@@ -21349,7 +21349,7 @@
         <v>65</v>
       </c>
       <c r="D51" s="1">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>239</v>
@@ -21375,7 +21375,7 @@
         <v>182</v>
       </c>
       <c r="D52" s="1">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>239</v>
@@ -21401,7 +21401,7 @@
         <v>182</v>
       </c>
       <c r="D53" s="1">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>239</v>
@@ -21427,7 +21427,7 @@
         <v>182</v>
       </c>
       <c r="D54" s="1">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>239</v>
@@ -21453,7 +21453,7 @@
         <v>249</v>
       </c>
       <c r="D55" s="1">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>239</v>
@@ -21479,7 +21479,7 @@
         <v>251</v>
       </c>
       <c r="D56" s="1">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>239</v>
@@ -21505,7 +21505,7 @@
         <v>182</v>
       </c>
       <c r="D57" s="1">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>239</v>
@@ -21531,7 +21531,7 @@
         <v>58</v>
       </c>
       <c r="D58" s="1">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>239</v>
@@ -21557,7 +21557,7 @@
         <v>182</v>
       </c>
       <c r="D59" s="1">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>239</v>
@@ -21583,7 +21583,7 @@
         <v>65</v>
       </c>
       <c r="D60" s="1">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>239</v>
@@ -21609,7 +21609,7 @@
         <v>251</v>
       </c>
       <c r="D61" s="1">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>239</v>
@@ -21635,7 +21635,7 @@
         <v>182</v>
       </c>
       <c r="D62" s="1">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>239</v>
@@ -21661,7 +21661,7 @@
         <v>251</v>
       </c>
       <c r="D63" s="1">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>239</v>

</xml_diff>

<commit_message>
New location for manual top up
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="2"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="7" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -3706,13 +3706,13 @@
     <t>Fever Facility</t>
   </si>
   <si>
+    <t>L1 ED</t>
+  </si>
+  <si>
     <t>ED X-Ray</t>
   </si>
   <si>
     <t>Room 1</t>
-  </si>
-  <si>
-    <t>L1 ED</t>
   </si>
   <si>
     <t>Room 2</t>
@@ -10112,8 +10112,12 @@
       <c r="E50" s="1" t="s">
         <v>1165</v>
       </c>
-      <c r="F50" s="1"/>
-      <c r="G50" s="1"/>
+      <c r="F50" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>1225</v>
+      </c>
       <c r="H50" s="1" t="s">
         <v>15</v>
       </c>
@@ -10135,16 +10139,16 @@
         <v>1118</v>
       </c>
       <c r="D51" s="1" t="s">
+        <v>1226</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>1227</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G51" s="1" t="s">
         <v>1225</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>1226</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>1227</v>
       </c>
       <c r="H51" s="1" t="s">
         <v>15</v>
@@ -10167,7 +10171,7 @@
         <v>1118</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>1228</v>
@@ -10176,7 +10180,7 @@
         <v>15</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>1227</v>
+        <v>1225</v>
       </c>
       <c r="H52" s="1" t="s">
         <v>15</v>
@@ -10199,7 +10203,7 @@
         <v>1118</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>1120</v>
@@ -10208,7 +10212,7 @@
         <v>15</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>1227</v>
+        <v>1225</v>
       </c>
       <c r="H53" s="1" t="s">
         <v>15</v>
@@ -10231,7 +10235,7 @@
         <v>1118</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>1229</v>

</xml_diff>